<commit_message>
Correction de l'export excel
</commit_message>
<xml_diff>
--- a/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
+++ b/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Appsdev\workspaces\santalina\src\main\webui\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seb/Documents/developpement-seb/santalina/src/main/resources/META-INF/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC285AD-44A3-4658-978A-AFBEB7E1D505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D38E2A-A81E-3345-BB16-B2D1E83D9AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
+    <workbookView xWindow="-100" yWindow="500" windowWidth="23260" windowHeight="13900" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
   </bookViews>
   <sheets>
     <sheet name="P1-1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'P1-1'!$A$1:$M$34</definedName>
   </definedNames>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -519,7 +519,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -778,6 +778,51 @@
       </top>
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -804,7 +849,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
@@ -932,25 +977,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="49" fontId="27" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="22" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -966,7 +993,31 @@
     <xf numFmtId="49" fontId="19" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="19" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="19" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="20" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="21" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1525,56 +1576,56 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="3.5546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="24.88671875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="3.5" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.1640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.1640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="8.33203125" style="2" customWidth="1"/>
     <col min="7" max="7" width="5" style="2" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" style="2" customWidth="1"/>
-    <col min="9" max="12" width="10.77734375" style="2" customWidth="1"/>
-    <col min="13" max="13" width="29.88671875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="3.44140625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="12.21875" style="2" customWidth="1"/>
-    <col min="16" max="16" width="9.109375" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" style="2"/>
+    <col min="9" max="12" width="10.83203125" style="2" customWidth="1"/>
+    <col min="13" max="13" width="29.83203125" style="2" customWidth="1"/>
+    <col min="14" max="14" width="3.5" style="2" customWidth="1"/>
+    <col min="15" max="15" width="12.1640625" style="2" customWidth="1"/>
+    <col min="16" max="16" width="9.1640625" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="60.75" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="54"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1">
       <c r="A2" s="3"/>
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="56" t="s">
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="50"/>
       <c r="M2" s="4" t="s">
         <v>2</v>
       </c>
@@ -1596,14 +1647,14 @@
     </row>
     <row r="4" spans="1:18" ht="41.25" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="57" t="s">
+      <c r="B4" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="51"/>
       <c r="H4" s="7" t="s">
         <v>4</v>
       </c>
@@ -1613,10 +1664,10 @@
       <c r="J4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="58" t="s">
+      <c r="K4" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="L4" s="58"/>
+      <c r="L4" s="52"/>
       <c r="M4" s="9" t="s">
         <v>8</v>
       </c>
@@ -1656,15 +1707,15 @@
       <c r="G6" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="59" t="s">
+      <c r="H6" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="59"/>
-      <c r="J6" s="59" t="s">
+      <c r="I6" s="47"/>
+      <c r="J6" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="59"/>
-      <c r="L6" s="59"/>
+      <c r="K6" s="47"/>
+      <c r="L6" s="47"/>
       <c r="M6" s="14" t="s">
         <v>17</v>
       </c>
@@ -1686,7 +1737,7 @@
       <c r="M7" s="18"/>
     </row>
     <row r="8" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A8" s="53">
+      <c r="A8" s="58">
         <v>1</v>
       </c>
       <c r="B8" s="19"/>
@@ -1695,19 +1746,19 @@
       <c r="E8" s="19"/>
       <c r="F8" s="20"/>
       <c r="G8" s="21"/>
-      <c r="H8" s="50" t="s">
+      <c r="H8" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="50" t="s">
+      <c r="I8" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="51" t="s">
+      <c r="J8" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="K8" s="51" t="s">
+      <c r="K8" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="51" t="s">
+      <c r="L8" s="53" t="s">
         <v>22</v>
       </c>
       <c r="M8" s="22" t="s">
@@ -1719,18 +1770,18 @@
       <c r="Q8" s="24"/>
     </row>
     <row r="9" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A9" s="53"/>
+      <c r="A9" s="58"/>
       <c r="B9" s="25"/>
       <c r="C9" s="25"/>
       <c r="D9" s="25"/>
       <c r="E9" s="25"/>
       <c r="F9" s="20"/>
       <c r="G9" s="21"/>
-      <c r="H9" s="50"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="51"/>
-      <c r="K9" s="51"/>
-      <c r="L9" s="51"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
+      <c r="J9" s="53"/>
+      <c r="K9" s="53"/>
+      <c r="L9" s="53"/>
       <c r="M9" s="22" t="s">
         <v>24</v>
       </c>
@@ -1740,18 +1791,18 @@
       <c r="Q9" s="24"/>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A10" s="53"/>
+      <c r="A10" s="58"/>
       <c r="B10" s="27"/>
       <c r="C10" s="27"/>
       <c r="D10" s="19"/>
       <c r="E10" s="19"/>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
-      <c r="H10" s="50"/>
-      <c r="I10" s="50"/>
-      <c r="J10" s="51"/>
-      <c r="K10" s="51"/>
-      <c r="L10" s="51"/>
+      <c r="H10" s="55"/>
+      <c r="I10" s="55"/>
+      <c r="J10" s="53"/>
+      <c r="K10" s="53"/>
+      <c r="L10" s="53"/>
       <c r="M10" s="22" t="s">
         <v>25</v>
       </c>
@@ -1762,27 +1813,27 @@
       <c r="R10" s="24"/>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A11" s="53"/>
+      <c r="A11" s="58"/>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="50"/>
-      <c r="J11" s="52" t="s">
+      <c r="H11" s="55"/>
+      <c r="I11" s="55"/>
+      <c r="J11" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="52"/>
-      <c r="L11" s="52"/>
+      <c r="K11" s="54"/>
+      <c r="L11" s="54"/>
       <c r="M11" s="28" t="s">
         <v>27</v>
       </c>
       <c r="R11" s="24"/>
     </row>
     <row r="12" spans="1:18" ht="9" customHeight="1">
-      <c r="A12" s="21"/>
+      <c r="A12" s="59"/>
       <c r="B12" s="29"/>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
@@ -1797,7 +1848,7 @@
       <c r="M12" s="31"/>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A13" s="53">
+      <c r="A13" s="58">
         <v>2</v>
       </c>
       <c r="B13" s="19"/>
@@ -1806,19 +1857,19 @@
       <c r="E13" s="19"/>
       <c r="F13" s="20"/>
       <c r="G13" s="21"/>
-      <c r="H13" s="50" t="s">
+      <c r="H13" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="50" t="s">
+      <c r="I13" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="51" t="s">
+      <c r="J13" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="K13" s="51" t="s">
+      <c r="K13" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L13" s="51" t="s">
+      <c r="L13" s="53" t="s">
         <v>22</v>
       </c>
       <c r="M13" s="22" t="s">
@@ -1831,18 +1882,18 @@
       <c r="R13" s="24"/>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A14" s="53"/>
+      <c r="A14" s="58"/>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="E14" s="25"/>
       <c r="F14" s="20"/>
       <c r="G14" s="21"/>
-      <c r="H14" s="50"/>
-      <c r="I14" s="50"/>
-      <c r="J14" s="51"/>
-      <c r="K14" s="51"/>
-      <c r="L14" s="51"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
+      <c r="J14" s="53"/>
+      <c r="K14" s="53"/>
+      <c r="L14" s="53"/>
       <c r="M14" s="22" t="s">
         <v>24</v>
       </c>
@@ -1852,18 +1903,18 @@
       <c r="R14" s="24"/>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A15" s="53"/>
+      <c r="A15" s="58"/>
       <c r="B15" s="25"/>
       <c r="C15" s="19"/>
       <c r="D15" s="25"/>
       <c r="E15" s="25"/>
       <c r="F15" s="21"/>
       <c r="G15" s="21"/>
-      <c r="H15" s="50"/>
-      <c r="I15" s="50"/>
-      <c r="J15" s="51"/>
-      <c r="K15" s="51"/>
-      <c r="L15" s="51"/>
+      <c r="H15" s="55"/>
+      <c r="I15" s="55"/>
+      <c r="J15" s="53"/>
+      <c r="K15" s="53"/>
+      <c r="L15" s="53"/>
       <c r="M15" s="22" t="s">
         <v>25</v>
       </c>
@@ -1873,20 +1924,20 @@
       <c r="R15" s="24"/>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A16" s="53"/>
+      <c r="A16" s="58"/>
       <c r="B16" s="21"/>
       <c r="C16" s="21"/>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
       <c r="F16" s="21"/>
       <c r="G16" s="21"/>
-      <c r="H16" s="50"/>
-      <c r="I16" s="50"/>
-      <c r="J16" s="52" t="s">
+      <c r="H16" s="55"/>
+      <c r="I16" s="55"/>
+      <c r="J16" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="K16" s="52"/>
-      <c r="L16" s="52"/>
+      <c r="K16" s="54"/>
+      <c r="L16" s="54"/>
       <c r="M16" s="28" t="s">
         <v>27</v>
       </c>
@@ -1895,7 +1946,7 @@
       <c r="P16" s="23"/>
     </row>
     <row r="17" spans="1:21" ht="9" customHeight="1">
-      <c r="A17" s="21"/>
+      <c r="A17" s="59"/>
       <c r="B17" s="29"/>
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
@@ -1912,7 +1963,7 @@
       <c r="O17" s="32"/>
     </row>
     <row r="18" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A18" s="49">
+      <c r="A18" s="60">
         <v>3</v>
       </c>
       <c r="B18" s="25"/>
@@ -1921,19 +1972,19 @@
       <c r="E18" s="19"/>
       <c r="F18" s="20"/>
       <c r="G18" s="21"/>
-      <c r="H18" s="50" t="s">
+      <c r="H18" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="50" t="s">
+      <c r="I18" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="51" t="s">
+      <c r="J18" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="K18" s="51" t="s">
+      <c r="K18" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L18" s="51" t="s">
+      <c r="L18" s="53" t="s">
         <v>22</v>
       </c>
       <c r="M18" s="22" t="s">
@@ -1945,18 +1996,18 @@
       <c r="R18" s="24"/>
     </row>
     <row r="19" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A19" s="49"/>
+      <c r="A19" s="60"/>
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
       <c r="D19" s="25"/>
       <c r="E19" s="25"/>
       <c r="F19" s="21"/>
       <c r="G19" s="21"/>
-      <c r="H19" s="50"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="51"/>
-      <c r="K19" s="51"/>
-      <c r="L19" s="51"/>
+      <c r="H19" s="55"/>
+      <c r="I19" s="55"/>
+      <c r="J19" s="53"/>
+      <c r="K19" s="53"/>
+      <c r="L19" s="53"/>
       <c r="M19" s="22" t="s">
         <v>24</v>
       </c>
@@ -1967,18 +2018,18 @@
       <c r="R19" s="24"/>
     </row>
     <row r="20" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A20" s="49"/>
+      <c r="A20" s="60"/>
       <c r="B20" s="25"/>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
       <c r="E20" s="25"/>
       <c r="F20" s="21"/>
       <c r="G20" s="21"/>
-      <c r="H20" s="50"/>
-      <c r="I20" s="50"/>
-      <c r="J20" s="51"/>
-      <c r="K20" s="51"/>
-      <c r="L20" s="51"/>
+      <c r="H20" s="55"/>
+      <c r="I20" s="55"/>
+      <c r="J20" s="53"/>
+      <c r="K20" s="53"/>
+      <c r="L20" s="53"/>
       <c r="M20" s="22" t="s">
         <v>25</v>
       </c>
@@ -1988,20 +2039,20 @@
       <c r="R20" s="24"/>
     </row>
     <row r="21" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A21" s="49"/>
+      <c r="A21" s="60"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
       <c r="G21" s="21"/>
-      <c r="H21" s="50"/>
-      <c r="I21" s="50"/>
-      <c r="J21" s="52" t="s">
+      <c r="H21" s="55"/>
+      <c r="I21" s="55"/>
+      <c r="J21" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="K21" s="52"/>
-      <c r="L21" s="52"/>
+      <c r="K21" s="54"/>
+      <c r="L21" s="54"/>
       <c r="M21" s="28" t="s">
         <v>27</v>
       </c>
@@ -2009,7 +2060,7 @@
       <c r="R21" s="24"/>
     </row>
     <row r="22" spans="1:21" ht="9" customHeight="1">
-      <c r="A22" s="21"/>
+      <c r="A22" s="59"/>
       <c r="B22" s="29"/>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
@@ -2025,7 +2076,7 @@
       <c r="R22" s="33"/>
     </row>
     <row r="23" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A23" s="49">
+      <c r="A23" s="60">
         <v>4</v>
       </c>
       <c r="B23" s="25"/>
@@ -2034,19 +2085,19 @@
       <c r="E23" s="19"/>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
-      <c r="H23" s="50" t="s">
+      <c r="H23" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="50" t="s">
+      <c r="I23" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="J23" s="51" t="s">
+      <c r="J23" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="51" t="s">
+      <c r="K23" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L23" s="51" t="s">
+      <c r="L23" s="53" t="s">
         <v>22</v>
       </c>
       <c r="M23" s="22" t="s">
@@ -2059,18 +2110,18 @@
       <c r="U23" s="33"/>
     </row>
     <row r="24" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A24" s="49"/>
+      <c r="A24" s="60"/>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
       <c r="D24" s="25"/>
       <c r="E24" s="25"/>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
-      <c r="H24" s="50"/>
-      <c r="I24" s="50"/>
-      <c r="J24" s="51"/>
-      <c r="K24" s="51"/>
-      <c r="L24" s="51"/>
+      <c r="H24" s="55"/>
+      <c r="I24" s="55"/>
+      <c r="J24" s="53"/>
+      <c r="K24" s="53"/>
+      <c r="L24" s="53"/>
       <c r="M24" s="22" t="s">
         <v>24</v>
       </c>
@@ -2080,18 +2131,18 @@
       <c r="R24" s="24"/>
     </row>
     <row r="25" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A25" s="49"/>
+      <c r="A25" s="60"/>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="D25" s="27"/>
       <c r="E25" s="27"/>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
-      <c r="H25" s="50"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="51"/>
-      <c r="K25" s="51"/>
-      <c r="L25" s="51"/>
+      <c r="H25" s="55"/>
+      <c r="I25" s="55"/>
+      <c r="J25" s="53"/>
+      <c r="K25" s="53"/>
+      <c r="L25" s="53"/>
       <c r="M25" s="22" t="s">
         <v>25</v>
       </c>
@@ -2100,20 +2151,20 @@
       <c r="P25" s="34"/>
     </row>
     <row r="26" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A26" s="49"/>
+      <c r="A26" s="60"/>
       <c r="B26" s="21"/>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
       <c r="E26" s="21"/>
       <c r="F26" s="21"/>
       <c r="G26" s="21"/>
-      <c r="H26" s="50"/>
-      <c r="I26" s="50"/>
-      <c r="J26" s="52" t="s">
+      <c r="H26" s="55"/>
+      <c r="I26" s="55"/>
+      <c r="J26" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="K26" s="52"/>
-      <c r="L26" s="52"/>
+      <c r="K26" s="54"/>
+      <c r="L26" s="54"/>
       <c r="M26" s="28" t="s">
         <v>27</v>
       </c>
@@ -2123,7 +2174,7 @@
       <c r="Q26" s="33"/>
     </row>
     <row r="27" spans="1:21" ht="9" customHeight="1">
-      <c r="A27" s="21"/>
+      <c r="A27" s="59"/>
       <c r="B27" s="29"/>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
@@ -2138,7 +2189,7 @@
       <c r="M27" s="31"/>
     </row>
     <row r="28" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A28" s="49">
+      <c r="A28" s="60">
         <v>5</v>
       </c>
       <c r="B28" s="25"/>
@@ -2147,19 +2198,19 @@
       <c r="E28" s="25"/>
       <c r="F28" s="21"/>
       <c r="G28" s="21"/>
-      <c r="H28" s="50" t="s">
+      <c r="H28" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="50" t="s">
+      <c r="I28" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="J28" s="51" t="s">
+      <c r="J28" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="K28" s="51" t="s">
+      <c r="K28" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L28" s="51" t="s">
+      <c r="L28" s="53" t="s">
         <v>22</v>
       </c>
       <c r="M28" s="22" t="s">
@@ -2170,18 +2221,18 @@
       <c r="P28" s="23"/>
     </row>
     <row r="29" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A29" s="49"/>
+      <c r="A29" s="60"/>
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
       <c r="E29" s="25"/>
       <c r="F29" s="20"/>
       <c r="G29" s="21"/>
-      <c r="H29" s="50"/>
-      <c r="I29" s="50"/>
-      <c r="J29" s="51"/>
-      <c r="K29" s="51"/>
-      <c r="L29" s="51"/>
+      <c r="H29" s="55"/>
+      <c r="I29" s="55"/>
+      <c r="J29" s="53"/>
+      <c r="K29" s="53"/>
+      <c r="L29" s="53"/>
       <c r="M29" s="22" t="s">
         <v>24</v>
       </c>
@@ -2190,18 +2241,18 @@
       <c r="P29" s="23"/>
     </row>
     <row r="30" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A30" s="49"/>
+      <c r="A30" s="60"/>
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
       <c r="D30" s="25"/>
       <c r="E30" s="25"/>
       <c r="F30" s="20"/>
       <c r="G30" s="21"/>
-      <c r="H30" s="50"/>
-      <c r="I30" s="50"/>
-      <c r="J30" s="51"/>
-      <c r="K30" s="51"/>
-      <c r="L30" s="51"/>
+      <c r="H30" s="55"/>
+      <c r="I30" s="55"/>
+      <c r="J30" s="53"/>
+      <c r="K30" s="53"/>
+      <c r="L30" s="53"/>
       <c r="M30" s="22" t="s">
         <v>25</v>
       </c>
@@ -2210,20 +2261,20 @@
       <c r="P30" s="23"/>
     </row>
     <row r="31" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A31" s="49"/>
+      <c r="A31" s="60"/>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
       <c r="D31" s="25"/>
       <c r="E31" s="25"/>
       <c r="F31" s="20"/>
       <c r="G31" s="21"/>
-      <c r="H31" s="50"/>
-      <c r="I31" s="50"/>
-      <c r="J31" s="52" t="s">
+      <c r="H31" s="55"/>
+      <c r="I31" s="55"/>
+      <c r="J31" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="K31" s="52"/>
-      <c r="L31" s="52"/>
+      <c r="K31" s="54"/>
+      <c r="L31" s="54"/>
       <c r="M31" s="28" t="s">
         <v>27</v>
       </c>
@@ -2232,7 +2283,7 @@
       <c r="P31" s="34"/>
     </row>
     <row r="32" spans="1:21" ht="18.75" hidden="1" customHeight="1">
-      <c r="A32" s="49"/>
+      <c r="A32" s="60"/>
       <c r="B32" s="35"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -2250,7 +2301,7 @@
       <c r="Q32" s="24"/>
     </row>
     <row r="33" spans="1:17" ht="18.75" hidden="1" customHeight="1">
-      <c r="A33" s="49"/>
+      <c r="A33" s="61"/>
       <c r="B33" s="35"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -2268,22 +2319,22 @@
     </row>
     <row r="34" spans="1:17" ht="36.75" customHeight="1">
       <c r="A34" s="21"/>
-      <c r="B34" s="47" t="s">
+      <c r="B34" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="47"/>
-      <c r="D34" s="47"/>
-      <c r="E34" s="47"/>
-      <c r="F34" s="47"/>
-      <c r="G34" s="47"/>
-      <c r="H34" s="47"/>
-      <c r="I34" s="48" t="s">
+      <c r="C34" s="56"/>
+      <c r="D34" s="56"/>
+      <c r="E34" s="56"/>
+      <c r="F34" s="56"/>
+      <c r="G34" s="56"/>
+      <c r="H34" s="56"/>
+      <c r="I34" s="57" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="48"/>
-      <c r="K34" s="48"/>
-      <c r="L34" s="48"/>
-      <c r="M34" s="48"/>
+      <c r="J34" s="57"/>
+      <c r="K34" s="57"/>
+      <c r="L34" s="57"/>
+      <c r="M34" s="57"/>
       <c r="Q34" s="33"/>
     </row>
     <row r="35" spans="1:17" ht="12.75" customHeight="1">
@@ -2309,13 +2360,29 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="B34:H34"/>
+    <mergeCell ref="I34:M34"/>
+    <mergeCell ref="A28:A33"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="I28:I31"/>
+    <mergeCell ref="J28:J30"/>
+    <mergeCell ref="K28:K30"/>
+    <mergeCell ref="L28:L30"/>
+    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="L23:L25"/>
+    <mergeCell ref="J26:L26"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="I18:I21"/>
+    <mergeCell ref="J18:J20"/>
+    <mergeCell ref="K18:K20"/>
+    <mergeCell ref="L18:L20"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="H23:H26"/>
+    <mergeCell ref="I23:I26"/>
+    <mergeCell ref="J23:J25"/>
+    <mergeCell ref="K23:K25"/>
     <mergeCell ref="L13:L15"/>
     <mergeCell ref="J16:L16"/>
     <mergeCell ref="A8:A11"/>
@@ -2330,33 +2397,17 @@
     <mergeCell ref="I13:I16"/>
     <mergeCell ref="J13:J15"/>
     <mergeCell ref="K13:K15"/>
-    <mergeCell ref="L23:L25"/>
-    <mergeCell ref="J26:L26"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="I18:I21"/>
-    <mergeCell ref="J18:J20"/>
-    <mergeCell ref="K18:K20"/>
-    <mergeCell ref="L18:L20"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="H23:H26"/>
-    <mergeCell ref="I23:I26"/>
-    <mergeCell ref="J23:J25"/>
-    <mergeCell ref="K23:K25"/>
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="I34:M34"/>
-    <mergeCell ref="A28:A33"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="I28:I31"/>
-    <mergeCell ref="J28:J30"/>
-    <mergeCell ref="K28:K30"/>
-    <mergeCell ref="L28:L30"/>
-    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="K4:L4"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19645669291338586" right="0.19645669291338586" top="0.11811023622047245" bottom="0.51181102362204722" header="0.11811023622047245" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="80" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -2367,11 +2418,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4F2601A-D0F9-4D66-91F1-48C323321E9D}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.77734375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="2"/>
+    <col min="1" max="5" width="11.83203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.1640625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">
@@ -2456,11 +2507,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24971601-4DEF-44A8-8017-6E23A38D615F}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.77734375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="2"/>
+    <col min="1" max="5" width="11.83203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.1640625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
Correction de l'export excel (#61)
</commit_message>
<xml_diff>
--- a/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
+++ b/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Appsdev\workspaces\santalina\src\main\webui\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seb/Documents/developpement-seb/santalina/src/main/resources/META-INF/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC285AD-44A3-4658-978A-AFBEB7E1D505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D38E2A-A81E-3345-BB16-B2D1E83D9AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
+    <workbookView xWindow="-100" yWindow="500" windowWidth="23260" windowHeight="13900" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
   </bookViews>
   <sheets>
     <sheet name="P1-1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'P1-1'!$A$1:$M$34</definedName>
   </definedNames>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -519,7 +519,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -778,6 +778,51 @@
       </top>
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -804,7 +849,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
@@ -932,25 +977,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="49" fontId="27" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="22" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -966,7 +993,31 @@
     <xf numFmtId="49" fontId="19" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="19" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="19" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="20" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="21" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1525,56 +1576,56 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="3.5546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="24.88671875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="3.5" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.1640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.1640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="8.33203125" style="2" customWidth="1"/>
     <col min="7" max="7" width="5" style="2" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" style="2" customWidth="1"/>
-    <col min="9" max="12" width="10.77734375" style="2" customWidth="1"/>
-    <col min="13" max="13" width="29.88671875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="3.44140625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="12.21875" style="2" customWidth="1"/>
-    <col min="16" max="16" width="9.109375" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" style="2"/>
+    <col min="9" max="12" width="10.83203125" style="2" customWidth="1"/>
+    <col min="13" max="13" width="29.83203125" style="2" customWidth="1"/>
+    <col min="14" max="14" width="3.5" style="2" customWidth="1"/>
+    <col min="15" max="15" width="12.1640625" style="2" customWidth="1"/>
+    <col min="16" max="16" width="9.1640625" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="60.75" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="54"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1">
       <c r="A2" s="3"/>
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="56" t="s">
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="50"/>
       <c r="M2" s="4" t="s">
         <v>2</v>
       </c>
@@ -1596,14 +1647,14 @@
     </row>
     <row r="4" spans="1:18" ht="41.25" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="57" t="s">
+      <c r="B4" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="51"/>
       <c r="H4" s="7" t="s">
         <v>4</v>
       </c>
@@ -1613,10 +1664,10 @@
       <c r="J4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="58" t="s">
+      <c r="K4" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="L4" s="58"/>
+      <c r="L4" s="52"/>
       <c r="M4" s="9" t="s">
         <v>8</v>
       </c>
@@ -1656,15 +1707,15 @@
       <c r="G6" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="59" t="s">
+      <c r="H6" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="59"/>
-      <c r="J6" s="59" t="s">
+      <c r="I6" s="47"/>
+      <c r="J6" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="59"/>
-      <c r="L6" s="59"/>
+      <c r="K6" s="47"/>
+      <c r="L6" s="47"/>
       <c r="M6" s="14" t="s">
         <v>17</v>
       </c>
@@ -1686,7 +1737,7 @@
       <c r="M7" s="18"/>
     </row>
     <row r="8" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A8" s="53">
+      <c r="A8" s="58">
         <v>1</v>
       </c>
       <c r="B8" s="19"/>
@@ -1695,19 +1746,19 @@
       <c r="E8" s="19"/>
       <c r="F8" s="20"/>
       <c r="G8" s="21"/>
-      <c r="H8" s="50" t="s">
+      <c r="H8" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="50" t="s">
+      <c r="I8" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="51" t="s">
+      <c r="J8" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="K8" s="51" t="s">
+      <c r="K8" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="51" t="s">
+      <c r="L8" s="53" t="s">
         <v>22</v>
       </c>
       <c r="M8" s="22" t="s">
@@ -1719,18 +1770,18 @@
       <c r="Q8" s="24"/>
     </row>
     <row r="9" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A9" s="53"/>
+      <c r="A9" s="58"/>
       <c r="B9" s="25"/>
       <c r="C9" s="25"/>
       <c r="D9" s="25"/>
       <c r="E9" s="25"/>
       <c r="F9" s="20"/>
       <c r="G9" s="21"/>
-      <c r="H9" s="50"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="51"/>
-      <c r="K9" s="51"/>
-      <c r="L9" s="51"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
+      <c r="J9" s="53"/>
+      <c r="K9" s="53"/>
+      <c r="L9" s="53"/>
       <c r="M9" s="22" t="s">
         <v>24</v>
       </c>
@@ -1740,18 +1791,18 @@
       <c r="Q9" s="24"/>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A10" s="53"/>
+      <c r="A10" s="58"/>
       <c r="B10" s="27"/>
       <c r="C10" s="27"/>
       <c r="D10" s="19"/>
       <c r="E10" s="19"/>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
-      <c r="H10" s="50"/>
-      <c r="I10" s="50"/>
-      <c r="J10" s="51"/>
-      <c r="K10" s="51"/>
-      <c r="L10" s="51"/>
+      <c r="H10" s="55"/>
+      <c r="I10" s="55"/>
+      <c r="J10" s="53"/>
+      <c r="K10" s="53"/>
+      <c r="L10" s="53"/>
       <c r="M10" s="22" t="s">
         <v>25</v>
       </c>
@@ -1762,27 +1813,27 @@
       <c r="R10" s="24"/>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A11" s="53"/>
+      <c r="A11" s="58"/>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="50"/>
-      <c r="J11" s="52" t="s">
+      <c r="H11" s="55"/>
+      <c r="I11" s="55"/>
+      <c r="J11" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="52"/>
-      <c r="L11" s="52"/>
+      <c r="K11" s="54"/>
+      <c r="L11" s="54"/>
       <c r="M11" s="28" t="s">
         <v>27</v>
       </c>
       <c r="R11" s="24"/>
     </row>
     <row r="12" spans="1:18" ht="9" customHeight="1">
-      <c r="A12" s="21"/>
+      <c r="A12" s="59"/>
       <c r="B12" s="29"/>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
@@ -1797,7 +1848,7 @@
       <c r="M12" s="31"/>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A13" s="53">
+      <c r="A13" s="58">
         <v>2</v>
       </c>
       <c r="B13" s="19"/>
@@ -1806,19 +1857,19 @@
       <c r="E13" s="19"/>
       <c r="F13" s="20"/>
       <c r="G13" s="21"/>
-      <c r="H13" s="50" t="s">
+      <c r="H13" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="50" t="s">
+      <c r="I13" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="51" t="s">
+      <c r="J13" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="K13" s="51" t="s">
+      <c r="K13" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L13" s="51" t="s">
+      <c r="L13" s="53" t="s">
         <v>22</v>
       </c>
       <c r="M13" s="22" t="s">
@@ -1831,18 +1882,18 @@
       <c r="R13" s="24"/>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A14" s="53"/>
+      <c r="A14" s="58"/>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="E14" s="25"/>
       <c r="F14" s="20"/>
       <c r="G14" s="21"/>
-      <c r="H14" s="50"/>
-      <c r="I14" s="50"/>
-      <c r="J14" s="51"/>
-      <c r="K14" s="51"/>
-      <c r="L14" s="51"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
+      <c r="J14" s="53"/>
+      <c r="K14" s="53"/>
+      <c r="L14" s="53"/>
       <c r="M14" s="22" t="s">
         <v>24</v>
       </c>
@@ -1852,18 +1903,18 @@
       <c r="R14" s="24"/>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A15" s="53"/>
+      <c r="A15" s="58"/>
       <c r="B15" s="25"/>
       <c r="C15" s="19"/>
       <c r="D15" s="25"/>
       <c r="E15" s="25"/>
       <c r="F15" s="21"/>
       <c r="G15" s="21"/>
-      <c r="H15" s="50"/>
-      <c r="I15" s="50"/>
-      <c r="J15" s="51"/>
-      <c r="K15" s="51"/>
-      <c r="L15" s="51"/>
+      <c r="H15" s="55"/>
+      <c r="I15" s="55"/>
+      <c r="J15" s="53"/>
+      <c r="K15" s="53"/>
+      <c r="L15" s="53"/>
       <c r="M15" s="22" t="s">
         <v>25</v>
       </c>
@@ -1873,20 +1924,20 @@
       <c r="R15" s="24"/>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A16" s="53"/>
+      <c r="A16" s="58"/>
       <c r="B16" s="21"/>
       <c r="C16" s="21"/>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
       <c r="F16" s="21"/>
       <c r="G16" s="21"/>
-      <c r="H16" s="50"/>
-      <c r="I16" s="50"/>
-      <c r="J16" s="52" t="s">
+      <c r="H16" s="55"/>
+      <c r="I16" s="55"/>
+      <c r="J16" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="K16" s="52"/>
-      <c r="L16" s="52"/>
+      <c r="K16" s="54"/>
+      <c r="L16" s="54"/>
       <c r="M16" s="28" t="s">
         <v>27</v>
       </c>
@@ -1895,7 +1946,7 @@
       <c r="P16" s="23"/>
     </row>
     <row r="17" spans="1:21" ht="9" customHeight="1">
-      <c r="A17" s="21"/>
+      <c r="A17" s="59"/>
       <c r="B17" s="29"/>
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
@@ -1912,7 +1963,7 @@
       <c r="O17" s="32"/>
     </row>
     <row r="18" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A18" s="49">
+      <c r="A18" s="60">
         <v>3</v>
       </c>
       <c r="B18" s="25"/>
@@ -1921,19 +1972,19 @@
       <c r="E18" s="19"/>
       <c r="F18" s="20"/>
       <c r="G18" s="21"/>
-      <c r="H18" s="50" t="s">
+      <c r="H18" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="50" t="s">
+      <c r="I18" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="51" t="s">
+      <c r="J18" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="K18" s="51" t="s">
+      <c r="K18" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L18" s="51" t="s">
+      <c r="L18" s="53" t="s">
         <v>22</v>
       </c>
       <c r="M18" s="22" t="s">
@@ -1945,18 +1996,18 @@
       <c r="R18" s="24"/>
     </row>
     <row r="19" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A19" s="49"/>
+      <c r="A19" s="60"/>
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
       <c r="D19" s="25"/>
       <c r="E19" s="25"/>
       <c r="F19" s="21"/>
       <c r="G19" s="21"/>
-      <c r="H19" s="50"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="51"/>
-      <c r="K19" s="51"/>
-      <c r="L19" s="51"/>
+      <c r="H19" s="55"/>
+      <c r="I19" s="55"/>
+      <c r="J19" s="53"/>
+      <c r="K19" s="53"/>
+      <c r="L19" s="53"/>
       <c r="M19" s="22" t="s">
         <v>24</v>
       </c>
@@ -1967,18 +2018,18 @@
       <c r="R19" s="24"/>
     </row>
     <row r="20" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A20" s="49"/>
+      <c r="A20" s="60"/>
       <c r="B20" s="25"/>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
       <c r="E20" s="25"/>
       <c r="F20" s="21"/>
       <c r="G20" s="21"/>
-      <c r="H20" s="50"/>
-      <c r="I20" s="50"/>
-      <c r="J20" s="51"/>
-      <c r="K20" s="51"/>
-      <c r="L20" s="51"/>
+      <c r="H20" s="55"/>
+      <c r="I20" s="55"/>
+      <c r="J20" s="53"/>
+      <c r="K20" s="53"/>
+      <c r="L20" s="53"/>
       <c r="M20" s="22" t="s">
         <v>25</v>
       </c>
@@ -1988,20 +2039,20 @@
       <c r="R20" s="24"/>
     </row>
     <row r="21" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A21" s="49"/>
+      <c r="A21" s="60"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
       <c r="G21" s="21"/>
-      <c r="H21" s="50"/>
-      <c r="I21" s="50"/>
-      <c r="J21" s="52" t="s">
+      <c r="H21" s="55"/>
+      <c r="I21" s="55"/>
+      <c r="J21" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="K21" s="52"/>
-      <c r="L21" s="52"/>
+      <c r="K21" s="54"/>
+      <c r="L21" s="54"/>
       <c r="M21" s="28" t="s">
         <v>27</v>
       </c>
@@ -2009,7 +2060,7 @@
       <c r="R21" s="24"/>
     </row>
     <row r="22" spans="1:21" ht="9" customHeight="1">
-      <c r="A22" s="21"/>
+      <c r="A22" s="59"/>
       <c r="B22" s="29"/>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
@@ -2025,7 +2076,7 @@
       <c r="R22" s="33"/>
     </row>
     <row r="23" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A23" s="49">
+      <c r="A23" s="60">
         <v>4</v>
       </c>
       <c r="B23" s="25"/>
@@ -2034,19 +2085,19 @@
       <c r="E23" s="19"/>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
-      <c r="H23" s="50" t="s">
+      <c r="H23" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="50" t="s">
+      <c r="I23" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="J23" s="51" t="s">
+      <c r="J23" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="51" t="s">
+      <c r="K23" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L23" s="51" t="s">
+      <c r="L23" s="53" t="s">
         <v>22</v>
       </c>
       <c r="M23" s="22" t="s">
@@ -2059,18 +2110,18 @@
       <c r="U23" s="33"/>
     </row>
     <row r="24" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A24" s="49"/>
+      <c r="A24" s="60"/>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
       <c r="D24" s="25"/>
       <c r="E24" s="25"/>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
-      <c r="H24" s="50"/>
-      <c r="I24" s="50"/>
-      <c r="J24" s="51"/>
-      <c r="K24" s="51"/>
-      <c r="L24" s="51"/>
+      <c r="H24" s="55"/>
+      <c r="I24" s="55"/>
+      <c r="J24" s="53"/>
+      <c r="K24" s="53"/>
+      <c r="L24" s="53"/>
       <c r="M24" s="22" t="s">
         <v>24</v>
       </c>
@@ -2080,18 +2131,18 @@
       <c r="R24" s="24"/>
     </row>
     <row r="25" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A25" s="49"/>
+      <c r="A25" s="60"/>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="D25" s="27"/>
       <c r="E25" s="27"/>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
-      <c r="H25" s="50"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="51"/>
-      <c r="K25" s="51"/>
-      <c r="L25" s="51"/>
+      <c r="H25" s="55"/>
+      <c r="I25" s="55"/>
+      <c r="J25" s="53"/>
+      <c r="K25" s="53"/>
+      <c r="L25" s="53"/>
       <c r="M25" s="22" t="s">
         <v>25</v>
       </c>
@@ -2100,20 +2151,20 @@
       <c r="P25" s="34"/>
     </row>
     <row r="26" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A26" s="49"/>
+      <c r="A26" s="60"/>
       <c r="B26" s="21"/>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
       <c r="E26" s="21"/>
       <c r="F26" s="21"/>
       <c r="G26" s="21"/>
-      <c r="H26" s="50"/>
-      <c r="I26" s="50"/>
-      <c r="J26" s="52" t="s">
+      <c r="H26" s="55"/>
+      <c r="I26" s="55"/>
+      <c r="J26" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="K26" s="52"/>
-      <c r="L26" s="52"/>
+      <c r="K26" s="54"/>
+      <c r="L26" s="54"/>
       <c r="M26" s="28" t="s">
         <v>27</v>
       </c>
@@ -2123,7 +2174,7 @@
       <c r="Q26" s="33"/>
     </row>
     <row r="27" spans="1:21" ht="9" customHeight="1">
-      <c r="A27" s="21"/>
+      <c r="A27" s="59"/>
       <c r="B27" s="29"/>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
@@ -2138,7 +2189,7 @@
       <c r="M27" s="31"/>
     </row>
     <row r="28" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A28" s="49">
+      <c r="A28" s="60">
         <v>5</v>
       </c>
       <c r="B28" s="25"/>
@@ -2147,19 +2198,19 @@
       <c r="E28" s="25"/>
       <c r="F28" s="21"/>
       <c r="G28" s="21"/>
-      <c r="H28" s="50" t="s">
+      <c r="H28" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="50" t="s">
+      <c r="I28" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="J28" s="51" t="s">
+      <c r="J28" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="K28" s="51" t="s">
+      <c r="K28" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="L28" s="51" t="s">
+      <c r="L28" s="53" t="s">
         <v>22</v>
       </c>
       <c r="M28" s="22" t="s">
@@ -2170,18 +2221,18 @@
       <c r="P28" s="23"/>
     </row>
     <row r="29" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A29" s="49"/>
+      <c r="A29" s="60"/>
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
       <c r="E29" s="25"/>
       <c r="F29" s="20"/>
       <c r="G29" s="21"/>
-      <c r="H29" s="50"/>
-      <c r="I29" s="50"/>
-      <c r="J29" s="51"/>
-      <c r="K29" s="51"/>
-      <c r="L29" s="51"/>
+      <c r="H29" s="55"/>
+      <c r="I29" s="55"/>
+      <c r="J29" s="53"/>
+      <c r="K29" s="53"/>
+      <c r="L29" s="53"/>
       <c r="M29" s="22" t="s">
         <v>24</v>
       </c>
@@ -2190,18 +2241,18 @@
       <c r="P29" s="23"/>
     </row>
     <row r="30" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A30" s="49"/>
+      <c r="A30" s="60"/>
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
       <c r="D30" s="25"/>
       <c r="E30" s="25"/>
       <c r="F30" s="20"/>
       <c r="G30" s="21"/>
-      <c r="H30" s="50"/>
-      <c r="I30" s="50"/>
-      <c r="J30" s="51"/>
-      <c r="K30" s="51"/>
-      <c r="L30" s="51"/>
+      <c r="H30" s="55"/>
+      <c r="I30" s="55"/>
+      <c r="J30" s="53"/>
+      <c r="K30" s="53"/>
+      <c r="L30" s="53"/>
       <c r="M30" s="22" t="s">
         <v>25</v>
       </c>
@@ -2210,20 +2261,20 @@
       <c r="P30" s="23"/>
     </row>
     <row r="31" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A31" s="49"/>
+      <c r="A31" s="60"/>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
       <c r="D31" s="25"/>
       <c r="E31" s="25"/>
       <c r="F31" s="20"/>
       <c r="G31" s="21"/>
-      <c r="H31" s="50"/>
-      <c r="I31" s="50"/>
-      <c r="J31" s="52" t="s">
+      <c r="H31" s="55"/>
+      <c r="I31" s="55"/>
+      <c r="J31" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="K31" s="52"/>
-      <c r="L31" s="52"/>
+      <c r="K31" s="54"/>
+      <c r="L31" s="54"/>
       <c r="M31" s="28" t="s">
         <v>27</v>
       </c>
@@ -2232,7 +2283,7 @@
       <c r="P31" s="34"/>
     </row>
     <row r="32" spans="1:21" ht="18.75" hidden="1" customHeight="1">
-      <c r="A32" s="49"/>
+      <c r="A32" s="60"/>
       <c r="B32" s="35"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -2250,7 +2301,7 @@
       <c r="Q32" s="24"/>
     </row>
     <row r="33" spans="1:17" ht="18.75" hidden="1" customHeight="1">
-      <c r="A33" s="49"/>
+      <c r="A33" s="61"/>
       <c r="B33" s="35"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -2268,22 +2319,22 @@
     </row>
     <row r="34" spans="1:17" ht="36.75" customHeight="1">
       <c r="A34" s="21"/>
-      <c r="B34" s="47" t="s">
+      <c r="B34" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="47"/>
-      <c r="D34" s="47"/>
-      <c r="E34" s="47"/>
-      <c r="F34" s="47"/>
-      <c r="G34" s="47"/>
-      <c r="H34" s="47"/>
-      <c r="I34" s="48" t="s">
+      <c r="C34" s="56"/>
+      <c r="D34" s="56"/>
+      <c r="E34" s="56"/>
+      <c r="F34" s="56"/>
+      <c r="G34" s="56"/>
+      <c r="H34" s="56"/>
+      <c r="I34" s="57" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="48"/>
-      <c r="K34" s="48"/>
-      <c r="L34" s="48"/>
-      <c r="M34" s="48"/>
+      <c r="J34" s="57"/>
+      <c r="K34" s="57"/>
+      <c r="L34" s="57"/>
+      <c r="M34" s="57"/>
       <c r="Q34" s="33"/>
     </row>
     <row r="35" spans="1:17" ht="12.75" customHeight="1">
@@ -2309,13 +2360,29 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="B34:H34"/>
+    <mergeCell ref="I34:M34"/>
+    <mergeCell ref="A28:A33"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="I28:I31"/>
+    <mergeCell ref="J28:J30"/>
+    <mergeCell ref="K28:K30"/>
+    <mergeCell ref="L28:L30"/>
+    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="L23:L25"/>
+    <mergeCell ref="J26:L26"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="I18:I21"/>
+    <mergeCell ref="J18:J20"/>
+    <mergeCell ref="K18:K20"/>
+    <mergeCell ref="L18:L20"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="H23:H26"/>
+    <mergeCell ref="I23:I26"/>
+    <mergeCell ref="J23:J25"/>
+    <mergeCell ref="K23:K25"/>
     <mergeCell ref="L13:L15"/>
     <mergeCell ref="J16:L16"/>
     <mergeCell ref="A8:A11"/>
@@ -2330,33 +2397,17 @@
     <mergeCell ref="I13:I16"/>
     <mergeCell ref="J13:J15"/>
     <mergeCell ref="K13:K15"/>
-    <mergeCell ref="L23:L25"/>
-    <mergeCell ref="J26:L26"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="I18:I21"/>
-    <mergeCell ref="J18:J20"/>
-    <mergeCell ref="K18:K20"/>
-    <mergeCell ref="L18:L20"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="H23:H26"/>
-    <mergeCell ref="I23:I26"/>
-    <mergeCell ref="J23:J25"/>
-    <mergeCell ref="K23:K25"/>
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="I34:M34"/>
-    <mergeCell ref="A28:A33"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="I28:I31"/>
-    <mergeCell ref="J28:J30"/>
-    <mergeCell ref="K28:K30"/>
-    <mergeCell ref="L28:L30"/>
-    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="K4:L4"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19645669291338586" right="0.19645669291338586" top="0.11811023622047245" bottom="0.51181102362204722" header="0.11811023622047245" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="80" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -2367,11 +2418,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4F2601A-D0F9-4D66-91F1-48C323321E9D}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.77734375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="2"/>
+    <col min="1" max="5" width="11.83203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.1640625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">
@@ -2456,11 +2507,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24971601-4DEF-44A8-8017-6E23A38D615F}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.77734375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="2"/>
+    <col min="1" max="5" width="11.83203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.1640625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
Modification hauteur du pool
</commit_message>
<xml_diff>
--- a/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
+++ b/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seb/Documents/developpement-seb/santalina/src/main/resources/META-INF/resources/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Appsdev\workspaces\santalina\src\main\webui\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D38E2A-A81E-3345-BB16-B2D1E83D9AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC285AD-44A3-4658-978A-AFBEB7E1D505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-100" yWindow="500" windowWidth="23260" windowHeight="13900" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
   </bookViews>
   <sheets>
     <sheet name="P1-1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'P1-1'!$A$1:$M$34</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -519,7 +519,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -781,51 +781,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFFFFFFF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -849,7 +804,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
@@ -977,7 +932,25 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="27" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -993,31 +966,7 @@
     <xf numFmtId="49" fontId="19" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="19" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="19" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="20" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="21" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="22" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1576,56 +1525,56 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="3.5" style="2" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.1640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11.83203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="11.1640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="3.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.88671875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" style="2" customWidth="1"/>
     <col min="6" max="6" width="8.33203125" style="2" customWidth="1"/>
     <col min="7" max="7" width="5" style="2" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" style="2" customWidth="1"/>
-    <col min="9" max="12" width="10.83203125" style="2" customWidth="1"/>
-    <col min="13" max="13" width="29.83203125" style="2" customWidth="1"/>
-    <col min="14" max="14" width="3.5" style="2" customWidth="1"/>
-    <col min="15" max="15" width="12.1640625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="9.1640625" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.1640625" style="2"/>
+    <col min="9" max="12" width="10.77734375" style="2" customWidth="1"/>
+    <col min="13" max="13" width="29.88671875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="3.44140625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="12.21875" style="2" customWidth="1"/>
+    <col min="16" max="16" width="9.109375" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="60.75" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
+      <c r="K1" s="54"/>
+      <c r="L1" s="54"/>
+      <c r="M1" s="54"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1">
       <c r="A2" s="3"/>
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="50" t="s">
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
-      <c r="L2" s="50"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
       <c r="M2" s="4" t="s">
         <v>2</v>
       </c>
@@ -1647,14 +1596,14 @@
     </row>
     <row r="4" spans="1:18" ht="41.25" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="51" t="s">
+      <c r="B4" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="51"/>
-      <c r="F4" s="51"/>
-      <c r="G4" s="51"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
       <c r="H4" s="7" t="s">
         <v>4</v>
       </c>
@@ -1664,10 +1613,10 @@
       <c r="J4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="52" t="s">
+      <c r="K4" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="L4" s="52"/>
+      <c r="L4" s="58"/>
       <c r="M4" s="9" t="s">
         <v>8</v>
       </c>
@@ -1707,15 +1656,15 @@
       <c r="G6" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="47" t="s">
+      <c r="H6" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47" t="s">
+      <c r="I6" s="59"/>
+      <c r="J6" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
+      <c r="K6" s="59"/>
+      <c r="L6" s="59"/>
       <c r="M6" s="14" t="s">
         <v>17</v>
       </c>
@@ -1737,7 +1686,7 @@
       <c r="M7" s="18"/>
     </row>
     <row r="8" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A8" s="58">
+      <c r="A8" s="53">
         <v>1</v>
       </c>
       <c r="B8" s="19"/>
@@ -1746,19 +1695,19 @@
       <c r="E8" s="19"/>
       <c r="F8" s="20"/>
       <c r="G8" s="21"/>
-      <c r="H8" s="55" t="s">
+      <c r="H8" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="55" t="s">
+      <c r="I8" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="53" t="s">
+      <c r="J8" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K8" s="53" t="s">
+      <c r="K8" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="53" t="s">
+      <c r="L8" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M8" s="22" t="s">
@@ -1770,18 +1719,18 @@
       <c r="Q8" s="24"/>
     </row>
     <row r="9" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A9" s="58"/>
+      <c r="A9" s="53"/>
       <c r="B9" s="25"/>
       <c r="C9" s="25"/>
       <c r="D9" s="25"/>
       <c r="E9" s="25"/>
       <c r="F9" s="20"/>
       <c r="G9" s="21"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
-      <c r="J9" s="53"/>
-      <c r="K9" s="53"/>
-      <c r="L9" s="53"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
       <c r="M9" s="22" t="s">
         <v>24</v>
       </c>
@@ -1791,18 +1740,18 @@
       <c r="Q9" s="24"/>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A10" s="58"/>
+      <c r="A10" s="53"/>
       <c r="B10" s="27"/>
       <c r="C10" s="27"/>
       <c r="D10" s="19"/>
       <c r="E10" s="19"/>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
-      <c r="J10" s="53"/>
-      <c r="K10" s="53"/>
-      <c r="L10" s="53"/>
+      <c r="H10" s="50"/>
+      <c r="I10" s="50"/>
+      <c r="J10" s="51"/>
+      <c r="K10" s="51"/>
+      <c r="L10" s="51"/>
       <c r="M10" s="22" t="s">
         <v>25</v>
       </c>
@@ -1813,27 +1762,27 @@
       <c r="R10" s="24"/>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A11" s="58"/>
+      <c r="A11" s="53"/>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
-      <c r="H11" s="55"/>
-      <c r="I11" s="55"/>
-      <c r="J11" s="54" t="s">
+      <c r="H11" s="50"/>
+      <c r="I11" s="50"/>
+      <c r="J11" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="54"/>
-      <c r="L11" s="54"/>
+      <c r="K11" s="52"/>
+      <c r="L11" s="52"/>
       <c r="M11" s="28" t="s">
         <v>27</v>
       </c>
       <c r="R11" s="24"/>
     </row>
     <row r="12" spans="1:18" ht="9" customHeight="1">
-      <c r="A12" s="59"/>
+      <c r="A12" s="21"/>
       <c r="B12" s="29"/>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
@@ -1848,7 +1797,7 @@
       <c r="M12" s="31"/>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A13" s="58">
+      <c r="A13" s="53">
         <v>2</v>
       </c>
       <c r="B13" s="19"/>
@@ -1857,19 +1806,19 @@
       <c r="E13" s="19"/>
       <c r="F13" s="20"/>
       <c r="G13" s="21"/>
-      <c r="H13" s="55" t="s">
+      <c r="H13" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="55" t="s">
+      <c r="I13" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="53" t="s">
+      <c r="J13" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K13" s="53" t="s">
+      <c r="K13" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L13" s="53" t="s">
+      <c r="L13" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M13" s="22" t="s">
@@ -1882,18 +1831,18 @@
       <c r="R13" s="24"/>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A14" s="58"/>
+      <c r="A14" s="53"/>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="E14" s="25"/>
       <c r="F14" s="20"/>
       <c r="G14" s="21"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
-      <c r="J14" s="53"/>
-      <c r="K14" s="53"/>
-      <c r="L14" s="53"/>
+      <c r="H14" s="50"/>
+      <c r="I14" s="50"/>
+      <c r="J14" s="51"/>
+      <c r="K14" s="51"/>
+      <c r="L14" s="51"/>
       <c r="M14" s="22" t="s">
         <v>24</v>
       </c>
@@ -1903,18 +1852,18 @@
       <c r="R14" s="24"/>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A15" s="58"/>
+      <c r="A15" s="53"/>
       <c r="B15" s="25"/>
       <c r="C15" s="19"/>
       <c r="D15" s="25"/>
       <c r="E15" s="25"/>
       <c r="F15" s="21"/>
       <c r="G15" s="21"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="55"/>
-      <c r="J15" s="53"/>
-      <c r="K15" s="53"/>
-      <c r="L15" s="53"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="50"/>
+      <c r="J15" s="51"/>
+      <c r="K15" s="51"/>
+      <c r="L15" s="51"/>
       <c r="M15" s="22" t="s">
         <v>25</v>
       </c>
@@ -1924,20 +1873,20 @@
       <c r="R15" s="24"/>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A16" s="58"/>
+      <c r="A16" s="53"/>
       <c r="B16" s="21"/>
       <c r="C16" s="21"/>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
       <c r="F16" s="21"/>
       <c r="G16" s="21"/>
-      <c r="H16" s="55"/>
-      <c r="I16" s="55"/>
-      <c r="J16" s="54" t="s">
+      <c r="H16" s="50"/>
+      <c r="I16" s="50"/>
+      <c r="J16" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K16" s="54"/>
-      <c r="L16" s="54"/>
+      <c r="K16" s="52"/>
+      <c r="L16" s="52"/>
       <c r="M16" s="28" t="s">
         <v>27</v>
       </c>
@@ -1946,7 +1895,7 @@
       <c r="P16" s="23"/>
     </row>
     <row r="17" spans="1:21" ht="9" customHeight="1">
-      <c r="A17" s="59"/>
+      <c r="A17" s="21"/>
       <c r="B17" s="29"/>
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
@@ -1963,7 +1912,7 @@
       <c r="O17" s="32"/>
     </row>
     <row r="18" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A18" s="60">
+      <c r="A18" s="49">
         <v>3</v>
       </c>
       <c r="B18" s="25"/>
@@ -1972,19 +1921,19 @@
       <c r="E18" s="19"/>
       <c r="F18" s="20"/>
       <c r="G18" s="21"/>
-      <c r="H18" s="55" t="s">
+      <c r="H18" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="55" t="s">
+      <c r="I18" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="53" t="s">
+      <c r="J18" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K18" s="53" t="s">
+      <c r="K18" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L18" s="53" t="s">
+      <c r="L18" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M18" s="22" t="s">
@@ -1996,18 +1945,18 @@
       <c r="R18" s="24"/>
     </row>
     <row r="19" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A19" s="60"/>
+      <c r="A19" s="49"/>
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
       <c r="D19" s="25"/>
       <c r="E19" s="25"/>
       <c r="F19" s="21"/>
       <c r="G19" s="21"/>
-      <c r="H19" s="55"/>
-      <c r="I19" s="55"/>
-      <c r="J19" s="53"/>
-      <c r="K19" s="53"/>
-      <c r="L19" s="53"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="51"/>
+      <c r="K19" s="51"/>
+      <c r="L19" s="51"/>
       <c r="M19" s="22" t="s">
         <v>24</v>
       </c>
@@ -2018,18 +1967,18 @@
       <c r="R19" s="24"/>
     </row>
     <row r="20" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A20" s="60"/>
+      <c r="A20" s="49"/>
       <c r="B20" s="25"/>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
       <c r="E20" s="25"/>
       <c r="F20" s="21"/>
       <c r="G20" s="21"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="55"/>
-      <c r="J20" s="53"/>
-      <c r="K20" s="53"/>
-      <c r="L20" s="53"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="50"/>
+      <c r="J20" s="51"/>
+      <c r="K20" s="51"/>
+      <c r="L20" s="51"/>
       <c r="M20" s="22" t="s">
         <v>25</v>
       </c>
@@ -2039,20 +1988,20 @@
       <c r="R20" s="24"/>
     </row>
     <row r="21" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A21" s="60"/>
+      <c r="A21" s="49"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
       <c r="G21" s="21"/>
-      <c r="H21" s="55"/>
-      <c r="I21" s="55"/>
-      <c r="J21" s="54" t="s">
+      <c r="H21" s="50"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K21" s="54"/>
-      <c r="L21" s="54"/>
+      <c r="K21" s="52"/>
+      <c r="L21" s="52"/>
       <c r="M21" s="28" t="s">
         <v>27</v>
       </c>
@@ -2060,7 +2009,7 @@
       <c r="R21" s="24"/>
     </row>
     <row r="22" spans="1:21" ht="9" customHeight="1">
-      <c r="A22" s="59"/>
+      <c r="A22" s="21"/>
       <c r="B22" s="29"/>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
@@ -2076,7 +2025,7 @@
       <c r="R22" s="33"/>
     </row>
     <row r="23" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A23" s="60">
+      <c r="A23" s="49">
         <v>4</v>
       </c>
       <c r="B23" s="25"/>
@@ -2085,19 +2034,19 @@
       <c r="E23" s="19"/>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
-      <c r="H23" s="55" t="s">
+      <c r="H23" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="55" t="s">
+      <c r="I23" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J23" s="53" t="s">
+      <c r="J23" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="53" t="s">
+      <c r="K23" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L23" s="53" t="s">
+      <c r="L23" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M23" s="22" t="s">
@@ -2110,18 +2059,18 @@
       <c r="U23" s="33"/>
     </row>
     <row r="24" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A24" s="60"/>
+      <c r="A24" s="49"/>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
       <c r="D24" s="25"/>
       <c r="E24" s="25"/>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
-      <c r="H24" s="55"/>
-      <c r="I24" s="55"/>
-      <c r="J24" s="53"/>
-      <c r="K24" s="53"/>
-      <c r="L24" s="53"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="50"/>
+      <c r="J24" s="51"/>
+      <c r="K24" s="51"/>
+      <c r="L24" s="51"/>
       <c r="M24" s="22" t="s">
         <v>24</v>
       </c>
@@ -2131,18 +2080,18 @@
       <c r="R24" s="24"/>
     </row>
     <row r="25" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A25" s="60"/>
+      <c r="A25" s="49"/>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="D25" s="27"/>
       <c r="E25" s="27"/>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
-      <c r="H25" s="55"/>
-      <c r="I25" s="55"/>
-      <c r="J25" s="53"/>
-      <c r="K25" s="53"/>
-      <c r="L25" s="53"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="51"/>
+      <c r="K25" s="51"/>
+      <c r="L25" s="51"/>
       <c r="M25" s="22" t="s">
         <v>25</v>
       </c>
@@ -2151,20 +2100,20 @@
       <c r="P25" s="34"/>
     </row>
     <row r="26" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A26" s="60"/>
+      <c r="A26" s="49"/>
       <c r="B26" s="21"/>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
       <c r="E26" s="21"/>
       <c r="F26" s="21"/>
       <c r="G26" s="21"/>
-      <c r="H26" s="55"/>
-      <c r="I26" s="55"/>
-      <c r="J26" s="54" t="s">
+      <c r="H26" s="50"/>
+      <c r="I26" s="50"/>
+      <c r="J26" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K26" s="54"/>
-      <c r="L26" s="54"/>
+      <c r="K26" s="52"/>
+      <c r="L26" s="52"/>
       <c r="M26" s="28" t="s">
         <v>27</v>
       </c>
@@ -2174,7 +2123,7 @@
       <c r="Q26" s="33"/>
     </row>
     <row r="27" spans="1:21" ht="9" customHeight="1">
-      <c r="A27" s="59"/>
+      <c r="A27" s="21"/>
       <c r="B27" s="29"/>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
@@ -2189,7 +2138,7 @@
       <c r="M27" s="31"/>
     </row>
     <row r="28" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A28" s="60">
+      <c r="A28" s="49">
         <v>5</v>
       </c>
       <c r="B28" s="25"/>
@@ -2198,19 +2147,19 @@
       <c r="E28" s="25"/>
       <c r="F28" s="21"/>
       <c r="G28" s="21"/>
-      <c r="H28" s="55" t="s">
+      <c r="H28" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="55" t="s">
+      <c r="I28" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J28" s="53" t="s">
+      <c r="J28" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K28" s="53" t="s">
+      <c r="K28" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L28" s="53" t="s">
+      <c r="L28" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M28" s="22" t="s">
@@ -2221,18 +2170,18 @@
       <c r="P28" s="23"/>
     </row>
     <row r="29" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A29" s="60"/>
+      <c r="A29" s="49"/>
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
       <c r="E29" s="25"/>
       <c r="F29" s="20"/>
       <c r="G29" s="21"/>
-      <c r="H29" s="55"/>
-      <c r="I29" s="55"/>
-      <c r="J29" s="53"/>
-      <c r="K29" s="53"/>
-      <c r="L29" s="53"/>
+      <c r="H29" s="50"/>
+      <c r="I29" s="50"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="51"/>
+      <c r="L29" s="51"/>
       <c r="M29" s="22" t="s">
         <v>24</v>
       </c>
@@ -2241,18 +2190,18 @@
       <c r="P29" s="23"/>
     </row>
     <row r="30" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A30" s="60"/>
+      <c r="A30" s="49"/>
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
       <c r="D30" s="25"/>
       <c r="E30" s="25"/>
       <c r="F30" s="20"/>
       <c r="G30" s="21"/>
-      <c r="H30" s="55"/>
-      <c r="I30" s="55"/>
-      <c r="J30" s="53"/>
-      <c r="K30" s="53"/>
-      <c r="L30" s="53"/>
+      <c r="H30" s="50"/>
+      <c r="I30" s="50"/>
+      <c r="J30" s="51"/>
+      <c r="K30" s="51"/>
+      <c r="L30" s="51"/>
       <c r="M30" s="22" t="s">
         <v>25</v>
       </c>
@@ -2261,20 +2210,20 @@
       <c r="P30" s="23"/>
     </row>
     <row r="31" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A31" s="60"/>
+      <c r="A31" s="49"/>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
       <c r="D31" s="25"/>
       <c r="E31" s="25"/>
       <c r="F31" s="20"/>
       <c r="G31" s="21"/>
-      <c r="H31" s="55"/>
-      <c r="I31" s="55"/>
-      <c r="J31" s="54" t="s">
+      <c r="H31" s="50"/>
+      <c r="I31" s="50"/>
+      <c r="J31" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K31" s="54"/>
-      <c r="L31" s="54"/>
+      <c r="K31" s="52"/>
+      <c r="L31" s="52"/>
       <c r="M31" s="28" t="s">
         <v>27</v>
       </c>
@@ -2283,7 +2232,7 @@
       <c r="P31" s="34"/>
     </row>
     <row r="32" spans="1:21" ht="18.75" hidden="1" customHeight="1">
-      <c r="A32" s="60"/>
+      <c r="A32" s="49"/>
       <c r="B32" s="35"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -2301,7 +2250,7 @@
       <c r="Q32" s="24"/>
     </row>
     <row r="33" spans="1:17" ht="18.75" hidden="1" customHeight="1">
-      <c r="A33" s="61"/>
+      <c r="A33" s="49"/>
       <c r="B33" s="35"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -2319,22 +2268,22 @@
     </row>
     <row r="34" spans="1:17" ht="36.75" customHeight="1">
       <c r="A34" s="21"/>
-      <c r="B34" s="56" t="s">
+      <c r="B34" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="56"/>
-      <c r="D34" s="56"/>
-      <c r="E34" s="56"/>
-      <c r="F34" s="56"/>
-      <c r="G34" s="56"/>
-      <c r="H34" s="56"/>
-      <c r="I34" s="57" t="s">
+      <c r="C34" s="47"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="47"/>
+      <c r="F34" s="47"/>
+      <c r="G34" s="47"/>
+      <c r="H34" s="47"/>
+      <c r="I34" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="57"/>
-      <c r="K34" s="57"/>
-      <c r="L34" s="57"/>
-      <c r="M34" s="57"/>
+      <c r="J34" s="48"/>
+      <c r="K34" s="48"/>
+      <c r="L34" s="48"/>
+      <c r="M34" s="48"/>
       <c r="Q34" s="33"/>
     </row>
     <row r="35" spans="1:17" ht="12.75" customHeight="1">
@@ -2360,15 +2309,27 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="I34:M34"/>
-    <mergeCell ref="A28:A33"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="I28:I31"/>
-    <mergeCell ref="J28:J30"/>
-    <mergeCell ref="K28:K30"/>
-    <mergeCell ref="L28:L30"/>
-    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="L13:L15"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="I8:I11"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="H13:H16"/>
+    <mergeCell ref="I13:I16"/>
+    <mergeCell ref="J13:J15"/>
+    <mergeCell ref="K13:K15"/>
     <mergeCell ref="L23:L25"/>
     <mergeCell ref="J26:L26"/>
     <mergeCell ref="A18:A21"/>
@@ -2383,31 +2344,19 @@
     <mergeCell ref="I23:I26"/>
     <mergeCell ref="J23:J25"/>
     <mergeCell ref="K23:K25"/>
-    <mergeCell ref="L13:L15"/>
-    <mergeCell ref="J16:L16"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="I8:I11"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="H13:H16"/>
-    <mergeCell ref="I13:I16"/>
-    <mergeCell ref="J13:J15"/>
-    <mergeCell ref="K13:K15"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="B34:H34"/>
+    <mergeCell ref="I34:M34"/>
+    <mergeCell ref="A28:A33"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="I28:I31"/>
+    <mergeCell ref="J28:J30"/>
+    <mergeCell ref="K28:K30"/>
+    <mergeCell ref="L28:L30"/>
+    <mergeCell ref="J31:L31"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19645669291338586" right="0.19645669291338586" top="0.11811023622047245" bottom="0.51181102362204722" header="0.11811023622047245" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="80" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -2418,11 +2367,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4F2601A-D0F9-4D66-91F1-48C323321E9D}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.83203125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.1640625" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.1640625" style="2"/>
+    <col min="1" max="5" width="11.77734375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">
@@ -2507,11 +2456,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24971601-4DEF-44A8-8017-6E23A38D615F}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.83203125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.1640625" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.1640625" style="2"/>
+    <col min="1" max="5" width="11.77734375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
Modification hauteur du pool (#62)
</commit_message>
<xml_diff>
--- a/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
+++ b/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seb/Documents/developpement-seb/santalina/src/main/resources/META-INF/resources/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Appsdev\workspaces\santalina\src\main\webui\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D38E2A-A81E-3345-BB16-B2D1E83D9AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC285AD-44A3-4658-978A-AFBEB7E1D505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-100" yWindow="500" windowWidth="23260" windowHeight="13900" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
   </bookViews>
   <sheets>
     <sheet name="P1-1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'P1-1'!$A$1:$M$34</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -519,7 +519,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -781,51 +781,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFFFFFFF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -849,7 +804,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
@@ -977,7 +932,25 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="27" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -993,31 +966,7 @@
     <xf numFmtId="49" fontId="19" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="19" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="19" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="20" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="21" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="22" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1576,56 +1525,56 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="3.5" style="2" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.1640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11.83203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="11.1640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="3.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.88671875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" style="2" customWidth="1"/>
     <col min="6" max="6" width="8.33203125" style="2" customWidth="1"/>
     <col min="7" max="7" width="5" style="2" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" style="2" customWidth="1"/>
-    <col min="9" max="12" width="10.83203125" style="2" customWidth="1"/>
-    <col min="13" max="13" width="29.83203125" style="2" customWidth="1"/>
-    <col min="14" max="14" width="3.5" style="2" customWidth="1"/>
-    <col min="15" max="15" width="12.1640625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="9.1640625" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.1640625" style="2"/>
+    <col min="9" max="12" width="10.77734375" style="2" customWidth="1"/>
+    <col min="13" max="13" width="29.88671875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="3.44140625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="12.21875" style="2" customWidth="1"/>
+    <col min="16" max="16" width="9.109375" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="60.75" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
+      <c r="K1" s="54"/>
+      <c r="L1" s="54"/>
+      <c r="M1" s="54"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1">
       <c r="A2" s="3"/>
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="50" t="s">
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
-      <c r="L2" s="50"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
       <c r="M2" s="4" t="s">
         <v>2</v>
       </c>
@@ -1647,14 +1596,14 @@
     </row>
     <row r="4" spans="1:18" ht="41.25" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="51" t="s">
+      <c r="B4" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="51"/>
-      <c r="F4" s="51"/>
-      <c r="G4" s="51"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
       <c r="H4" s="7" t="s">
         <v>4</v>
       </c>
@@ -1664,10 +1613,10 @@
       <c r="J4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="52" t="s">
+      <c r="K4" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="L4" s="52"/>
+      <c r="L4" s="58"/>
       <c r="M4" s="9" t="s">
         <v>8</v>
       </c>
@@ -1707,15 +1656,15 @@
       <c r="G6" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="47" t="s">
+      <c r="H6" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47" t="s">
+      <c r="I6" s="59"/>
+      <c r="J6" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
+      <c r="K6" s="59"/>
+      <c r="L6" s="59"/>
       <c r="M6" s="14" t="s">
         <v>17</v>
       </c>
@@ -1737,7 +1686,7 @@
       <c r="M7" s="18"/>
     </row>
     <row r="8" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A8" s="58">
+      <c r="A8" s="53">
         <v>1</v>
       </c>
       <c r="B8" s="19"/>
@@ -1746,19 +1695,19 @@
       <c r="E8" s="19"/>
       <c r="F8" s="20"/>
       <c r="G8" s="21"/>
-      <c r="H8" s="55" t="s">
+      <c r="H8" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="55" t="s">
+      <c r="I8" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="53" t="s">
+      <c r="J8" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K8" s="53" t="s">
+      <c r="K8" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="53" t="s">
+      <c r="L8" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M8" s="22" t="s">
@@ -1770,18 +1719,18 @@
       <c r="Q8" s="24"/>
     </row>
     <row r="9" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A9" s="58"/>
+      <c r="A9" s="53"/>
       <c r="B9" s="25"/>
       <c r="C9" s="25"/>
       <c r="D9" s="25"/>
       <c r="E9" s="25"/>
       <c r="F9" s="20"/>
       <c r="G9" s="21"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
-      <c r="J9" s="53"/>
-      <c r="K9" s="53"/>
-      <c r="L9" s="53"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
       <c r="M9" s="22" t="s">
         <v>24</v>
       </c>
@@ -1791,18 +1740,18 @@
       <c r="Q9" s="24"/>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A10" s="58"/>
+      <c r="A10" s="53"/>
       <c r="B10" s="27"/>
       <c r="C10" s="27"/>
       <c r="D10" s="19"/>
       <c r="E10" s="19"/>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
-      <c r="J10" s="53"/>
-      <c r="K10" s="53"/>
-      <c r="L10" s="53"/>
+      <c r="H10" s="50"/>
+      <c r="I10" s="50"/>
+      <c r="J10" s="51"/>
+      <c r="K10" s="51"/>
+      <c r="L10" s="51"/>
       <c r="M10" s="22" t="s">
         <v>25</v>
       </c>
@@ -1813,27 +1762,27 @@
       <c r="R10" s="24"/>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A11" s="58"/>
+      <c r="A11" s="53"/>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
-      <c r="H11" s="55"/>
-      <c r="I11" s="55"/>
-      <c r="J11" s="54" t="s">
+      <c r="H11" s="50"/>
+      <c r="I11" s="50"/>
+      <c r="J11" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="54"/>
-      <c r="L11" s="54"/>
+      <c r="K11" s="52"/>
+      <c r="L11" s="52"/>
       <c r="M11" s="28" t="s">
         <v>27</v>
       </c>
       <c r="R11" s="24"/>
     </row>
     <row r="12" spans="1:18" ht="9" customHeight="1">
-      <c r="A12" s="59"/>
+      <c r="A12" s="21"/>
       <c r="B12" s="29"/>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
@@ -1848,7 +1797,7 @@
       <c r="M12" s="31"/>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A13" s="58">
+      <c r="A13" s="53">
         <v>2</v>
       </c>
       <c r="B13" s="19"/>
@@ -1857,19 +1806,19 @@
       <c r="E13" s="19"/>
       <c r="F13" s="20"/>
       <c r="G13" s="21"/>
-      <c r="H13" s="55" t="s">
+      <c r="H13" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="55" t="s">
+      <c r="I13" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="53" t="s">
+      <c r="J13" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K13" s="53" t="s">
+      <c r="K13" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L13" s="53" t="s">
+      <c r="L13" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M13" s="22" t="s">
@@ -1882,18 +1831,18 @@
       <c r="R13" s="24"/>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A14" s="58"/>
+      <c r="A14" s="53"/>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="E14" s="25"/>
       <c r="F14" s="20"/>
       <c r="G14" s="21"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
-      <c r="J14" s="53"/>
-      <c r="K14" s="53"/>
-      <c r="L14" s="53"/>
+      <c r="H14" s="50"/>
+      <c r="I14" s="50"/>
+      <c r="J14" s="51"/>
+      <c r="K14" s="51"/>
+      <c r="L14" s="51"/>
       <c r="M14" s="22" t="s">
         <v>24</v>
       </c>
@@ -1903,18 +1852,18 @@
       <c r="R14" s="24"/>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A15" s="58"/>
+      <c r="A15" s="53"/>
       <c r="B15" s="25"/>
       <c r="C15" s="19"/>
       <c r="D15" s="25"/>
       <c r="E15" s="25"/>
       <c r="F15" s="21"/>
       <c r="G15" s="21"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="55"/>
-      <c r="J15" s="53"/>
-      <c r="K15" s="53"/>
-      <c r="L15" s="53"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="50"/>
+      <c r="J15" s="51"/>
+      <c r="K15" s="51"/>
+      <c r="L15" s="51"/>
       <c r="M15" s="22" t="s">
         <v>25</v>
       </c>
@@ -1924,20 +1873,20 @@
       <c r="R15" s="24"/>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A16" s="58"/>
+      <c r="A16" s="53"/>
       <c r="B16" s="21"/>
       <c r="C16" s="21"/>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
       <c r="F16" s="21"/>
       <c r="G16" s="21"/>
-      <c r="H16" s="55"/>
-      <c r="I16" s="55"/>
-      <c r="J16" s="54" t="s">
+      <c r="H16" s="50"/>
+      <c r="I16" s="50"/>
+      <c r="J16" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K16" s="54"/>
-      <c r="L16" s="54"/>
+      <c r="K16" s="52"/>
+      <c r="L16" s="52"/>
       <c r="M16" s="28" t="s">
         <v>27</v>
       </c>
@@ -1946,7 +1895,7 @@
       <c r="P16" s="23"/>
     </row>
     <row r="17" spans="1:21" ht="9" customHeight="1">
-      <c r="A17" s="59"/>
+      <c r="A17" s="21"/>
       <c r="B17" s="29"/>
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
@@ -1963,7 +1912,7 @@
       <c r="O17" s="32"/>
     </row>
     <row r="18" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A18" s="60">
+      <c r="A18" s="49">
         <v>3</v>
       </c>
       <c r="B18" s="25"/>
@@ -1972,19 +1921,19 @@
       <c r="E18" s="19"/>
       <c r="F18" s="20"/>
       <c r="G18" s="21"/>
-      <c r="H18" s="55" t="s">
+      <c r="H18" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="55" t="s">
+      <c r="I18" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="53" t="s">
+      <c r="J18" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K18" s="53" t="s">
+      <c r="K18" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L18" s="53" t="s">
+      <c r="L18" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M18" s="22" t="s">
@@ -1996,18 +1945,18 @@
       <c r="R18" s="24"/>
     </row>
     <row r="19" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A19" s="60"/>
+      <c r="A19" s="49"/>
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
       <c r="D19" s="25"/>
       <c r="E19" s="25"/>
       <c r="F19" s="21"/>
       <c r="G19" s="21"/>
-      <c r="H19" s="55"/>
-      <c r="I19" s="55"/>
-      <c r="J19" s="53"/>
-      <c r="K19" s="53"/>
-      <c r="L19" s="53"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="51"/>
+      <c r="K19" s="51"/>
+      <c r="L19" s="51"/>
       <c r="M19" s="22" t="s">
         <v>24</v>
       </c>
@@ -2018,18 +1967,18 @@
       <c r="R19" s="24"/>
     </row>
     <row r="20" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A20" s="60"/>
+      <c r="A20" s="49"/>
       <c r="B20" s="25"/>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
       <c r="E20" s="25"/>
       <c r="F20" s="21"/>
       <c r="G20" s="21"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="55"/>
-      <c r="J20" s="53"/>
-      <c r="K20" s="53"/>
-      <c r="L20" s="53"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="50"/>
+      <c r="J20" s="51"/>
+      <c r="K20" s="51"/>
+      <c r="L20" s="51"/>
       <c r="M20" s="22" t="s">
         <v>25</v>
       </c>
@@ -2039,20 +1988,20 @@
       <c r="R20" s="24"/>
     </row>
     <row r="21" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A21" s="60"/>
+      <c r="A21" s="49"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
       <c r="G21" s="21"/>
-      <c r="H21" s="55"/>
-      <c r="I21" s="55"/>
-      <c r="J21" s="54" t="s">
+      <c r="H21" s="50"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K21" s="54"/>
-      <c r="L21" s="54"/>
+      <c r="K21" s="52"/>
+      <c r="L21" s="52"/>
       <c r="M21" s="28" t="s">
         <v>27</v>
       </c>
@@ -2060,7 +2009,7 @@
       <c r="R21" s="24"/>
     </row>
     <row r="22" spans="1:21" ht="9" customHeight="1">
-      <c r="A22" s="59"/>
+      <c r="A22" s="21"/>
       <c r="B22" s="29"/>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
@@ -2076,7 +2025,7 @@
       <c r="R22" s="33"/>
     </row>
     <row r="23" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A23" s="60">
+      <c r="A23" s="49">
         <v>4</v>
       </c>
       <c r="B23" s="25"/>
@@ -2085,19 +2034,19 @@
       <c r="E23" s="19"/>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
-      <c r="H23" s="55" t="s">
+      <c r="H23" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="55" t="s">
+      <c r="I23" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J23" s="53" t="s">
+      <c r="J23" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="53" t="s">
+      <c r="K23" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L23" s="53" t="s">
+      <c r="L23" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M23" s="22" t="s">
@@ -2110,18 +2059,18 @@
       <c r="U23" s="33"/>
     </row>
     <row r="24" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A24" s="60"/>
+      <c r="A24" s="49"/>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
       <c r="D24" s="25"/>
       <c r="E24" s="25"/>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
-      <c r="H24" s="55"/>
-      <c r="I24" s="55"/>
-      <c r="J24" s="53"/>
-      <c r="K24" s="53"/>
-      <c r="L24" s="53"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="50"/>
+      <c r="J24" s="51"/>
+      <c r="K24" s="51"/>
+      <c r="L24" s="51"/>
       <c r="M24" s="22" t="s">
         <v>24</v>
       </c>
@@ -2131,18 +2080,18 @@
       <c r="R24" s="24"/>
     </row>
     <row r="25" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A25" s="60"/>
+      <c r="A25" s="49"/>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="D25" s="27"/>
       <c r="E25" s="27"/>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
-      <c r="H25" s="55"/>
-      <c r="I25" s="55"/>
-      <c r="J25" s="53"/>
-      <c r="K25" s="53"/>
-      <c r="L25" s="53"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="51"/>
+      <c r="K25" s="51"/>
+      <c r="L25" s="51"/>
       <c r="M25" s="22" t="s">
         <v>25</v>
       </c>
@@ -2151,20 +2100,20 @@
       <c r="P25" s="34"/>
     </row>
     <row r="26" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A26" s="60"/>
+      <c r="A26" s="49"/>
       <c r="B26" s="21"/>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
       <c r="E26" s="21"/>
       <c r="F26" s="21"/>
       <c r="G26" s="21"/>
-      <c r="H26" s="55"/>
-      <c r="I26" s="55"/>
-      <c r="J26" s="54" t="s">
+      <c r="H26" s="50"/>
+      <c r="I26" s="50"/>
+      <c r="J26" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K26" s="54"/>
-      <c r="L26" s="54"/>
+      <c r="K26" s="52"/>
+      <c r="L26" s="52"/>
       <c r="M26" s="28" t="s">
         <v>27</v>
       </c>
@@ -2174,7 +2123,7 @@
       <c r="Q26" s="33"/>
     </row>
     <row r="27" spans="1:21" ht="9" customHeight="1">
-      <c r="A27" s="59"/>
+      <c r="A27" s="21"/>
       <c r="B27" s="29"/>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
@@ -2189,7 +2138,7 @@
       <c r="M27" s="31"/>
     </row>
     <row r="28" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A28" s="60">
+      <c r="A28" s="49">
         <v>5</v>
       </c>
       <c r="B28" s="25"/>
@@ -2198,19 +2147,19 @@
       <c r="E28" s="25"/>
       <c r="F28" s="21"/>
       <c r="G28" s="21"/>
-      <c r="H28" s="55" t="s">
+      <c r="H28" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="55" t="s">
+      <c r="I28" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J28" s="53" t="s">
+      <c r="J28" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K28" s="53" t="s">
+      <c r="K28" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L28" s="53" t="s">
+      <c r="L28" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M28" s="22" t="s">
@@ -2221,18 +2170,18 @@
       <c r="P28" s="23"/>
     </row>
     <row r="29" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A29" s="60"/>
+      <c r="A29" s="49"/>
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
       <c r="E29" s="25"/>
       <c r="F29" s="20"/>
       <c r="G29" s="21"/>
-      <c r="H29" s="55"/>
-      <c r="I29" s="55"/>
-      <c r="J29" s="53"/>
-      <c r="K29" s="53"/>
-      <c r="L29" s="53"/>
+      <c r="H29" s="50"/>
+      <c r="I29" s="50"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="51"/>
+      <c r="L29" s="51"/>
       <c r="M29" s="22" t="s">
         <v>24</v>
       </c>
@@ -2241,18 +2190,18 @@
       <c r="P29" s="23"/>
     </row>
     <row r="30" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A30" s="60"/>
+      <c r="A30" s="49"/>
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
       <c r="D30" s="25"/>
       <c r="E30" s="25"/>
       <c r="F30" s="20"/>
       <c r="G30" s="21"/>
-      <c r="H30" s="55"/>
-      <c r="I30" s="55"/>
-      <c r="J30" s="53"/>
-      <c r="K30" s="53"/>
-      <c r="L30" s="53"/>
+      <c r="H30" s="50"/>
+      <c r="I30" s="50"/>
+      <c r="J30" s="51"/>
+      <c r="K30" s="51"/>
+      <c r="L30" s="51"/>
       <c r="M30" s="22" t="s">
         <v>25</v>
       </c>
@@ -2261,20 +2210,20 @@
       <c r="P30" s="23"/>
     </row>
     <row r="31" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A31" s="60"/>
+      <c r="A31" s="49"/>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
       <c r="D31" s="25"/>
       <c r="E31" s="25"/>
       <c r="F31" s="20"/>
       <c r="G31" s="21"/>
-      <c r="H31" s="55"/>
-      <c r="I31" s="55"/>
-      <c r="J31" s="54" t="s">
+      <c r="H31" s="50"/>
+      <c r="I31" s="50"/>
+      <c r="J31" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K31" s="54"/>
-      <c r="L31" s="54"/>
+      <c r="K31" s="52"/>
+      <c r="L31" s="52"/>
       <c r="M31" s="28" t="s">
         <v>27</v>
       </c>
@@ -2283,7 +2232,7 @@
       <c r="P31" s="34"/>
     </row>
     <row r="32" spans="1:21" ht="18.75" hidden="1" customHeight="1">
-      <c r="A32" s="60"/>
+      <c r="A32" s="49"/>
       <c r="B32" s="35"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -2301,7 +2250,7 @@
       <c r="Q32" s="24"/>
     </row>
     <row r="33" spans="1:17" ht="18.75" hidden="1" customHeight="1">
-      <c r="A33" s="61"/>
+      <c r="A33" s="49"/>
       <c r="B33" s="35"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -2319,22 +2268,22 @@
     </row>
     <row r="34" spans="1:17" ht="36.75" customHeight="1">
       <c r="A34" s="21"/>
-      <c r="B34" s="56" t="s">
+      <c r="B34" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="56"/>
-      <c r="D34" s="56"/>
-      <c r="E34" s="56"/>
-      <c r="F34" s="56"/>
-      <c r="G34" s="56"/>
-      <c r="H34" s="56"/>
-      <c r="I34" s="57" t="s">
+      <c r="C34" s="47"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="47"/>
+      <c r="F34" s="47"/>
+      <c r="G34" s="47"/>
+      <c r="H34" s="47"/>
+      <c r="I34" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="57"/>
-      <c r="K34" s="57"/>
-      <c r="L34" s="57"/>
-      <c r="M34" s="57"/>
+      <c r="J34" s="48"/>
+      <c r="K34" s="48"/>
+      <c r="L34" s="48"/>
+      <c r="M34" s="48"/>
       <c r="Q34" s="33"/>
     </row>
     <row r="35" spans="1:17" ht="12.75" customHeight="1">
@@ -2360,15 +2309,27 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="I34:M34"/>
-    <mergeCell ref="A28:A33"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="I28:I31"/>
-    <mergeCell ref="J28:J30"/>
-    <mergeCell ref="K28:K30"/>
-    <mergeCell ref="L28:L30"/>
-    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="L13:L15"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="I8:I11"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="H13:H16"/>
+    <mergeCell ref="I13:I16"/>
+    <mergeCell ref="J13:J15"/>
+    <mergeCell ref="K13:K15"/>
     <mergeCell ref="L23:L25"/>
     <mergeCell ref="J26:L26"/>
     <mergeCell ref="A18:A21"/>
@@ -2383,31 +2344,19 @@
     <mergeCell ref="I23:I26"/>
     <mergeCell ref="J23:J25"/>
     <mergeCell ref="K23:K25"/>
-    <mergeCell ref="L13:L15"/>
-    <mergeCell ref="J16:L16"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="I8:I11"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="H13:H16"/>
-    <mergeCell ref="I13:I16"/>
-    <mergeCell ref="J13:J15"/>
-    <mergeCell ref="K13:K15"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="B34:H34"/>
+    <mergeCell ref="I34:M34"/>
+    <mergeCell ref="A28:A33"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="I28:I31"/>
+    <mergeCell ref="J28:J30"/>
+    <mergeCell ref="K28:K30"/>
+    <mergeCell ref="L28:L30"/>
+    <mergeCell ref="J31:L31"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19645669291338586" right="0.19645669291338586" top="0.11811023622047245" bottom="0.51181102362204722" header="0.11811023622047245" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="80" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -2418,11 +2367,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4F2601A-D0F9-4D66-91F1-48C323321E9D}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.83203125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.1640625" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.1640625" style="2"/>
+    <col min="1" max="5" width="11.77734375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">
@@ -2507,11 +2456,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24971601-4DEF-44A8-8017-6E23A38D615F}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.83203125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.1640625" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.1640625" style="2"/>
+    <col min="1" max="5" width="11.77734375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
Changement des bordures du fichier excel
</commit_message>
<xml_diff>
--- a/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
+++ b/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seb/Documents/developpement-seb/santalina.nosync/src/main/resources/META-INF/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75A0A89-D7E6-584E-BB4D-1EB83FE17F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E92A8EF-2349-4541-9286-45C0952DBEDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="13900" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'P1-1'!$A$1:$M$34</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -519,7 +519,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -793,6 +793,21 @@
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
       </bottom>
       <diagonal/>
     </border>
@@ -849,7 +864,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
@@ -999,6 +1014,9 @@
     <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1008,16 +1026,16 @@
     <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="19" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="20" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="21" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="19" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="20" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="21" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="22" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1576,22 +1594,22 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="3.5" style="2" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.1640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11.83203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="11.1640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="8.33203125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="3.59765625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.796875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.19921875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.796875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.19921875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="8.3984375" style="2" customWidth="1"/>
     <col min="7" max="7" width="5" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="2" customWidth="1"/>
-    <col min="9" max="12" width="10.83203125" style="2" customWidth="1"/>
-    <col min="13" max="13" width="29.83203125" style="2" customWidth="1"/>
-    <col min="14" max="14" width="3.5" style="2" customWidth="1"/>
-    <col min="15" max="15" width="12.1640625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="9.1640625" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.1640625" style="2"/>
+    <col min="8" max="8" width="12.3984375" style="2" customWidth="1"/>
+    <col min="9" max="12" width="10.796875" style="2" customWidth="1"/>
+    <col min="13" max="13" width="29.796875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="3.3984375" style="2" customWidth="1"/>
+    <col min="15" max="15" width="12.19921875" style="2" customWidth="1"/>
+    <col min="16" max="16" width="9.19921875" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.19921875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="60.75" customHeight="1">
@@ -1737,7 +1755,7 @@
       <c r="M7" s="18"/>
     </row>
     <row r="8" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A8" s="58">
+      <c r="A8" s="55">
         <v>1</v>
       </c>
       <c r="B8" s="19"/>
@@ -1746,10 +1764,10 @@
       <c r="E8" s="19"/>
       <c r="F8" s="20"/>
       <c r="G8" s="21"/>
-      <c r="H8" s="55" t="s">
+      <c r="H8" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="55" t="s">
+      <c r="I8" s="56" t="s">
         <v>19</v>
       </c>
       <c r="J8" s="53" t="s">
@@ -1770,15 +1788,15 @@
       <c r="Q8" s="24"/>
     </row>
     <row r="9" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A9" s="58"/>
+      <c r="A9" s="55"/>
       <c r="B9" s="25"/>
       <c r="C9" s="25"/>
       <c r="D9" s="25"/>
       <c r="E9" s="25"/>
       <c r="F9" s="20"/>
       <c r="G9" s="21"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="56"/>
       <c r="J9" s="53"/>
       <c r="K9" s="53"/>
       <c r="L9" s="53"/>
@@ -1791,15 +1809,15 @@
       <c r="Q9" s="24"/>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A10" s="58"/>
+      <c r="A10" s="55"/>
       <c r="B10" s="27"/>
       <c r="C10" s="27"/>
       <c r="D10" s="19"/>
       <c r="E10" s="19"/>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
+      <c r="H10" s="56"/>
+      <c r="I10" s="56"/>
       <c r="J10" s="53"/>
       <c r="K10" s="53"/>
       <c r="L10" s="53"/>
@@ -1813,15 +1831,15 @@
       <c r="R10" s="24"/>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A11" s="58"/>
+      <c r="A11" s="55"/>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
-      <c r="H11" s="55"/>
-      <c r="I11" s="55"/>
+      <c r="H11" s="56"/>
+      <c r="I11" s="56"/>
       <c r="J11" s="54" t="s">
         <v>26</v>
       </c>
@@ -1833,7 +1851,7 @@
       <c r="R11" s="24"/>
     </row>
     <row r="12" spans="1:18" ht="9" customHeight="1">
-      <c r="A12" s="59"/>
+      <c r="A12" s="21"/>
       <c r="B12" s="29"/>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
@@ -1848,7 +1866,7 @@
       <c r="M12" s="31"/>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A13" s="58">
+      <c r="A13" s="55">
         <v>2</v>
       </c>
       <c r="B13" s="19"/>
@@ -1857,10 +1875,10 @@
       <c r="E13" s="19"/>
       <c r="F13" s="20"/>
       <c r="G13" s="21"/>
-      <c r="H13" s="55" t="s">
+      <c r="H13" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="55" t="s">
+      <c r="I13" s="56" t="s">
         <v>19</v>
       </c>
       <c r="J13" s="53" t="s">
@@ -1882,15 +1900,15 @@
       <c r="R13" s="24"/>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A14" s="58"/>
+      <c r="A14" s="55"/>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="E14" s="25"/>
       <c r="F14" s="20"/>
       <c r="G14" s="21"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
+      <c r="H14" s="56"/>
+      <c r="I14" s="56"/>
       <c r="J14" s="53"/>
       <c r="K14" s="53"/>
       <c r="L14" s="53"/>
@@ -1903,15 +1921,15 @@
       <c r="R14" s="24"/>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A15" s="58"/>
+      <c r="A15" s="55"/>
       <c r="B15" s="25"/>
       <c r="C15" s="19"/>
       <c r="D15" s="25"/>
       <c r="E15" s="25"/>
       <c r="F15" s="21"/>
       <c r="G15" s="21"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="55"/>
+      <c r="H15" s="56"/>
+      <c r="I15" s="56"/>
       <c r="J15" s="53"/>
       <c r="K15" s="53"/>
       <c r="L15" s="53"/>
@@ -1924,15 +1942,15 @@
       <c r="R15" s="24"/>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A16" s="58"/>
+      <c r="A16" s="55"/>
       <c r="B16" s="21"/>
       <c r="C16" s="21"/>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
       <c r="F16" s="21"/>
       <c r="G16" s="21"/>
-      <c r="H16" s="55"/>
-      <c r="I16" s="55"/>
+      <c r="H16" s="56"/>
+      <c r="I16" s="56"/>
       <c r="J16" s="54" t="s">
         <v>26</v>
       </c>
@@ -1946,7 +1964,7 @@
       <c r="P16" s="23"/>
     </row>
     <row r="17" spans="1:21" ht="9" customHeight="1">
-      <c r="A17" s="59"/>
+      <c r="A17" s="21"/>
       <c r="B17" s="29"/>
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
@@ -1963,7 +1981,7 @@
       <c r="O17" s="32"/>
     </row>
     <row r="18" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A18" s="60">
+      <c r="A18" s="59">
         <v>3</v>
       </c>
       <c r="B18" s="25"/>
@@ -1972,10 +1990,10 @@
       <c r="E18" s="19"/>
       <c r="F18" s="20"/>
       <c r="G18" s="21"/>
-      <c r="H18" s="55" t="s">
+      <c r="H18" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="55" t="s">
+      <c r="I18" s="56" t="s">
         <v>19</v>
       </c>
       <c r="J18" s="53" t="s">
@@ -2003,8 +2021,8 @@
       <c r="E19" s="25"/>
       <c r="F19" s="21"/>
       <c r="G19" s="21"/>
-      <c r="H19" s="55"/>
-      <c r="I19" s="55"/>
+      <c r="H19" s="56"/>
+      <c r="I19" s="56"/>
       <c r="J19" s="53"/>
       <c r="K19" s="53"/>
       <c r="L19" s="53"/>
@@ -2025,8 +2043,8 @@
       <c r="E20" s="25"/>
       <c r="F20" s="21"/>
       <c r="G20" s="21"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="55"/>
+      <c r="H20" s="56"/>
+      <c r="I20" s="56"/>
       <c r="J20" s="53"/>
       <c r="K20" s="53"/>
       <c r="L20" s="53"/>
@@ -2046,8 +2064,8 @@
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
       <c r="G21" s="21"/>
-      <c r="H21" s="55"/>
-      <c r="I21" s="55"/>
+      <c r="H21" s="56"/>
+      <c r="I21" s="56"/>
       <c r="J21" s="54" t="s">
         <v>26</v>
       </c>
@@ -2060,7 +2078,7 @@
       <c r="R21" s="24"/>
     </row>
     <row r="22" spans="1:21" ht="9" customHeight="1">
-      <c r="A22" s="59"/>
+      <c r="A22" s="61"/>
       <c r="B22" s="29"/>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
@@ -2085,10 +2103,10 @@
       <c r="E23" s="19"/>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
-      <c r="H23" s="55" t="s">
+      <c r="H23" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="55" t="s">
+      <c r="I23" s="56" t="s">
         <v>19</v>
       </c>
       <c r="J23" s="53" t="s">
@@ -2117,8 +2135,8 @@
       <c r="E24" s="25"/>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
-      <c r="H24" s="55"/>
-      <c r="I24" s="55"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="56"/>
       <c r="J24" s="53"/>
       <c r="K24" s="53"/>
       <c r="L24" s="53"/>
@@ -2138,8 +2156,8 @@
       <c r="E25" s="27"/>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
-      <c r="H25" s="55"/>
-      <c r="I25" s="55"/>
+      <c r="H25" s="56"/>
+      <c r="I25" s="56"/>
       <c r="J25" s="53"/>
       <c r="K25" s="53"/>
       <c r="L25" s="53"/>
@@ -2158,8 +2176,8 @@
       <c r="E26" s="21"/>
       <c r="F26" s="21"/>
       <c r="G26" s="21"/>
-      <c r="H26" s="55"/>
-      <c r="I26" s="55"/>
+      <c r="H26" s="56"/>
+      <c r="I26" s="56"/>
       <c r="J26" s="54" t="s">
         <v>26</v>
       </c>
@@ -2174,7 +2192,7 @@
       <c r="Q26" s="33"/>
     </row>
     <row r="27" spans="1:21" ht="9" customHeight="1">
-      <c r="A27" s="59"/>
+      <c r="A27" s="61"/>
       <c r="B27" s="29"/>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
@@ -2198,10 +2216,10 @@
       <c r="E28" s="25"/>
       <c r="F28" s="21"/>
       <c r="G28" s="21"/>
-      <c r="H28" s="55" t="s">
+      <c r="H28" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="55" t="s">
+      <c r="I28" s="56" t="s">
         <v>19</v>
       </c>
       <c r="J28" s="53" t="s">
@@ -2228,8 +2246,8 @@
       <c r="E29" s="25"/>
       <c r="F29" s="20"/>
       <c r="G29" s="21"/>
-      <c r="H29" s="55"/>
-      <c r="I29" s="55"/>
+      <c r="H29" s="56"/>
+      <c r="I29" s="56"/>
       <c r="J29" s="53"/>
       <c r="K29" s="53"/>
       <c r="L29" s="53"/>
@@ -2248,8 +2266,8 @@
       <c r="E30" s="25"/>
       <c r="F30" s="20"/>
       <c r="G30" s="21"/>
-      <c r="H30" s="55"/>
-      <c r="I30" s="55"/>
+      <c r="H30" s="56"/>
+      <c r="I30" s="56"/>
       <c r="J30" s="53"/>
       <c r="K30" s="53"/>
       <c r="L30" s="53"/>
@@ -2268,8 +2286,8 @@
       <c r="E31" s="25"/>
       <c r="F31" s="20"/>
       <c r="G31" s="21"/>
-      <c r="H31" s="55"/>
-      <c r="I31" s="55"/>
+      <c r="H31" s="56"/>
+      <c r="I31" s="56"/>
       <c r="J31" s="54" t="s">
         <v>26</v>
       </c>
@@ -2301,7 +2319,7 @@
       <c r="Q32" s="24"/>
     </row>
     <row r="33" spans="1:17" ht="18.75" hidden="1" customHeight="1">
-      <c r="A33" s="61"/>
+      <c r="A33" s="62"/>
       <c r="B33" s="35"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -2319,22 +2337,22 @@
     </row>
     <row r="34" spans="1:17" ht="36.75" customHeight="1">
       <c r="A34" s="21"/>
-      <c r="B34" s="56" t="s">
+      <c r="B34" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="56"/>
-      <c r="D34" s="56"/>
-      <c r="E34" s="56"/>
-      <c r="F34" s="56"/>
-      <c r="G34" s="56"/>
-      <c r="H34" s="56"/>
-      <c r="I34" s="57" t="s">
+      <c r="C34" s="57"/>
+      <c r="D34" s="57"/>
+      <c r="E34" s="57"/>
+      <c r="F34" s="57"/>
+      <c r="G34" s="57"/>
+      <c r="H34" s="57"/>
+      <c r="I34" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="57"/>
-      <c r="K34" s="57"/>
-      <c r="L34" s="57"/>
-      <c r="M34" s="57"/>
+      <c r="J34" s="58"/>
+      <c r="K34" s="58"/>
+      <c r="L34" s="58"/>
+      <c r="M34" s="58"/>
       <c r="Q34" s="33"/>
     </row>
     <row r="35" spans="1:17" ht="12.75" customHeight="1">
@@ -2407,7 +2425,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19645669291338586" right="0.19645669291338586" top="0.11811023622047245" bottom="0.51181102362204722" header="0.11811023622047245" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="80" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="92" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -2418,11 +2436,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4F2601A-D0F9-4D66-91F1-48C323321E9D}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.83203125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.1640625" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.1640625" style="2"/>
+    <col min="1" max="5" width="11.796875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.19921875" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.19921875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">
@@ -2507,11 +2525,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24971601-4DEF-44A8-8017-6E23A38D615F}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.83203125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.1640625" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.1640625" style="2"/>
+    <col min="1" max="5" width="11.796875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.19921875" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.19921875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
Retour arriere sur l'organisation de palanquée revient sur la vue en cours
</commit_message>
<xml_diff>
--- a/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
+++ b/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seb/Documents/developpement-seb/santalina.nosync/src/main/resources/META-INF/resources/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Appsdev\workspaces\santalina\src\main\webui\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E92A8EF-2349-4541-9286-45C0952DBEDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC285AD-44A3-4658-978A-AFBEB7E1D505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="13900" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
   </bookViews>
   <sheets>
     <sheet name="P1-1" sheetId="1" r:id="rId1"/>
@@ -519,7 +519,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -781,66 +781,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFFFFFFF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFFFFFFF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -864,7 +804,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
@@ -992,7 +932,25 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="7" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="27" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1008,34 +966,7 @@
     <xf numFmtId="49" fontId="19" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="28" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="20" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="21" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="19" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="22" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="22" fillId="9" borderId="3" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1594,56 +1525,56 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="3.59765625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="24.796875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.19921875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11.796875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="11.19921875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="8.3984375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="3.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.88671875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="8.33203125" style="2" customWidth="1"/>
     <col min="7" max="7" width="5" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12.3984375" style="2" customWidth="1"/>
-    <col min="9" max="12" width="10.796875" style="2" customWidth="1"/>
-    <col min="13" max="13" width="29.796875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="3.3984375" style="2" customWidth="1"/>
-    <col min="15" max="15" width="12.19921875" style="2" customWidth="1"/>
-    <col min="16" max="16" width="9.19921875" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.19921875" style="2"/>
+    <col min="8" max="8" width="12.33203125" style="2" customWidth="1"/>
+    <col min="9" max="12" width="10.77734375" style="2" customWidth="1"/>
+    <col min="13" max="13" width="29.88671875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="3.44140625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="12.21875" style="2" customWidth="1"/>
+    <col min="16" max="16" width="9.109375" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="60.75" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
+      <c r="K1" s="54"/>
+      <c r="L1" s="54"/>
+      <c r="M1" s="54"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1">
       <c r="A2" s="3"/>
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="50" t="s">
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
-      <c r="L2" s="50"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
       <c r="M2" s="4" t="s">
         <v>2</v>
       </c>
@@ -1665,14 +1596,14 @@
     </row>
     <row r="4" spans="1:18" ht="41.25" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="51" t="s">
+      <c r="B4" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="51"/>
-      <c r="F4" s="51"/>
-      <c r="G4" s="51"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
       <c r="H4" s="7" t="s">
         <v>4</v>
       </c>
@@ -1682,10 +1613,10 @@
       <c r="J4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="52" t="s">
+      <c r="K4" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="L4" s="52"/>
+      <c r="L4" s="58"/>
       <c r="M4" s="9" t="s">
         <v>8</v>
       </c>
@@ -1725,15 +1656,15 @@
       <c r="G6" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="47" t="s">
+      <c r="H6" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47" t="s">
+      <c r="I6" s="59"/>
+      <c r="J6" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
+      <c r="K6" s="59"/>
+      <c r="L6" s="59"/>
       <c r="M6" s="14" t="s">
         <v>17</v>
       </c>
@@ -1755,7 +1686,7 @@
       <c r="M7" s="18"/>
     </row>
     <row r="8" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A8" s="55">
+      <c r="A8" s="53">
         <v>1</v>
       </c>
       <c r="B8" s="19"/>
@@ -1764,19 +1695,19 @@
       <c r="E8" s="19"/>
       <c r="F8" s="20"/>
       <c r="G8" s="21"/>
-      <c r="H8" s="56" t="s">
+      <c r="H8" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="56" t="s">
+      <c r="I8" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="53" t="s">
+      <c r="J8" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K8" s="53" t="s">
+      <c r="K8" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="53" t="s">
+      <c r="L8" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M8" s="22" t="s">
@@ -1788,18 +1719,18 @@
       <c r="Q8" s="24"/>
     </row>
     <row r="9" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A9" s="55"/>
+      <c r="A9" s="53"/>
       <c r="B9" s="25"/>
       <c r="C9" s="25"/>
       <c r="D9" s="25"/>
       <c r="E9" s="25"/>
       <c r="F9" s="20"/>
       <c r="G9" s="21"/>
-      <c r="H9" s="56"/>
-      <c r="I9" s="56"/>
-      <c r="J9" s="53"/>
-      <c r="K9" s="53"/>
-      <c r="L9" s="53"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
       <c r="M9" s="22" t="s">
         <v>24</v>
       </c>
@@ -1809,18 +1740,18 @@
       <c r="Q9" s="24"/>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A10" s="55"/>
+      <c r="A10" s="53"/>
       <c r="B10" s="27"/>
       <c r="C10" s="27"/>
       <c r="D10" s="19"/>
       <c r="E10" s="19"/>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
-      <c r="H10" s="56"/>
-      <c r="I10" s="56"/>
-      <c r="J10" s="53"/>
-      <c r="K10" s="53"/>
-      <c r="L10" s="53"/>
+      <c r="H10" s="50"/>
+      <c r="I10" s="50"/>
+      <c r="J10" s="51"/>
+      <c r="K10" s="51"/>
+      <c r="L10" s="51"/>
       <c r="M10" s="22" t="s">
         <v>25</v>
       </c>
@@ -1831,20 +1762,20 @@
       <c r="R10" s="24"/>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A11" s="55"/>
+      <c r="A11" s="53"/>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
-      <c r="H11" s="56"/>
-      <c r="I11" s="56"/>
-      <c r="J11" s="54" t="s">
+      <c r="H11" s="50"/>
+      <c r="I11" s="50"/>
+      <c r="J11" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="54"/>
-      <c r="L11" s="54"/>
+      <c r="K11" s="52"/>
+      <c r="L11" s="52"/>
       <c r="M11" s="28" t="s">
         <v>27</v>
       </c>
@@ -1866,7 +1797,7 @@
       <c r="M12" s="31"/>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A13" s="55">
+      <c r="A13" s="53">
         <v>2</v>
       </c>
       <c r="B13" s="19"/>
@@ -1875,19 +1806,19 @@
       <c r="E13" s="19"/>
       <c r="F13" s="20"/>
       <c r="G13" s="21"/>
-      <c r="H13" s="56" t="s">
+      <c r="H13" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="56" t="s">
+      <c r="I13" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="53" t="s">
+      <c r="J13" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K13" s="53" t="s">
+      <c r="K13" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L13" s="53" t="s">
+      <c r="L13" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M13" s="22" t="s">
@@ -1900,18 +1831,18 @@
       <c r="R13" s="24"/>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A14" s="55"/>
+      <c r="A14" s="53"/>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="E14" s="25"/>
       <c r="F14" s="20"/>
       <c r="G14" s="21"/>
-      <c r="H14" s="56"/>
-      <c r="I14" s="56"/>
-      <c r="J14" s="53"/>
-      <c r="K14" s="53"/>
-      <c r="L14" s="53"/>
+      <c r="H14" s="50"/>
+      <c r="I14" s="50"/>
+      <c r="J14" s="51"/>
+      <c r="K14" s="51"/>
+      <c r="L14" s="51"/>
       <c r="M14" s="22" t="s">
         <v>24</v>
       </c>
@@ -1921,18 +1852,18 @@
       <c r="R14" s="24"/>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A15" s="55"/>
+      <c r="A15" s="53"/>
       <c r="B15" s="25"/>
       <c r="C15" s="19"/>
       <c r="D15" s="25"/>
       <c r="E15" s="25"/>
       <c r="F15" s="21"/>
       <c r="G15" s="21"/>
-      <c r="H15" s="56"/>
-      <c r="I15" s="56"/>
-      <c r="J15" s="53"/>
-      <c r="K15" s="53"/>
-      <c r="L15" s="53"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="50"/>
+      <c r="J15" s="51"/>
+      <c r="K15" s="51"/>
+      <c r="L15" s="51"/>
       <c r="M15" s="22" t="s">
         <v>25</v>
       </c>
@@ -1942,20 +1873,20 @@
       <c r="R15" s="24"/>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A16" s="55"/>
+      <c r="A16" s="53"/>
       <c r="B16" s="21"/>
       <c r="C16" s="21"/>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
       <c r="F16" s="21"/>
       <c r="G16" s="21"/>
-      <c r="H16" s="56"/>
-      <c r="I16" s="56"/>
-      <c r="J16" s="54" t="s">
+      <c r="H16" s="50"/>
+      <c r="I16" s="50"/>
+      <c r="J16" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K16" s="54"/>
-      <c r="L16" s="54"/>
+      <c r="K16" s="52"/>
+      <c r="L16" s="52"/>
       <c r="M16" s="28" t="s">
         <v>27</v>
       </c>
@@ -1981,7 +1912,7 @@
       <c r="O17" s="32"/>
     </row>
     <row r="18" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A18" s="59">
+      <c r="A18" s="49">
         <v>3</v>
       </c>
       <c r="B18" s="25"/>
@@ -1990,19 +1921,19 @@
       <c r="E18" s="19"/>
       <c r="F18" s="20"/>
       <c r="G18" s="21"/>
-      <c r="H18" s="56" t="s">
+      <c r="H18" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="56" t="s">
+      <c r="I18" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="53" t="s">
+      <c r="J18" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K18" s="53" t="s">
+      <c r="K18" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L18" s="53" t="s">
+      <c r="L18" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M18" s="22" t="s">
@@ -2014,18 +1945,18 @@
       <c r="R18" s="24"/>
     </row>
     <row r="19" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A19" s="60"/>
+      <c r="A19" s="49"/>
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
       <c r="D19" s="25"/>
       <c r="E19" s="25"/>
       <c r="F19" s="21"/>
       <c r="G19" s="21"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="56"/>
-      <c r="J19" s="53"/>
-      <c r="K19" s="53"/>
-      <c r="L19" s="53"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="51"/>
+      <c r="K19" s="51"/>
+      <c r="L19" s="51"/>
       <c r="M19" s="22" t="s">
         <v>24</v>
       </c>
@@ -2036,18 +1967,18 @@
       <c r="R19" s="24"/>
     </row>
     <row r="20" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A20" s="60"/>
+      <c r="A20" s="49"/>
       <c r="B20" s="25"/>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
       <c r="E20" s="25"/>
       <c r="F20" s="21"/>
       <c r="G20" s="21"/>
-      <c r="H20" s="56"/>
-      <c r="I20" s="56"/>
-      <c r="J20" s="53"/>
-      <c r="K20" s="53"/>
-      <c r="L20" s="53"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="50"/>
+      <c r="J20" s="51"/>
+      <c r="K20" s="51"/>
+      <c r="L20" s="51"/>
       <c r="M20" s="22" t="s">
         <v>25</v>
       </c>
@@ -2057,20 +1988,20 @@
       <c r="R20" s="24"/>
     </row>
     <row r="21" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A21" s="60"/>
+      <c r="A21" s="49"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
       <c r="G21" s="21"/>
-      <c r="H21" s="56"/>
-      <c r="I21" s="56"/>
-      <c r="J21" s="54" t="s">
+      <c r="H21" s="50"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K21" s="54"/>
-      <c r="L21" s="54"/>
+      <c r="K21" s="52"/>
+      <c r="L21" s="52"/>
       <c r="M21" s="28" t="s">
         <v>27</v>
       </c>
@@ -2078,7 +2009,7 @@
       <c r="R21" s="24"/>
     </row>
     <row r="22" spans="1:21" ht="9" customHeight="1">
-      <c r="A22" s="61"/>
+      <c r="A22" s="21"/>
       <c r="B22" s="29"/>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
@@ -2094,7 +2025,7 @@
       <c r="R22" s="33"/>
     </row>
     <row r="23" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A23" s="60">
+      <c r="A23" s="49">
         <v>4</v>
       </c>
       <c r="B23" s="25"/>
@@ -2103,19 +2034,19 @@
       <c r="E23" s="19"/>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
-      <c r="H23" s="56" t="s">
+      <c r="H23" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="56" t="s">
+      <c r="I23" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J23" s="53" t="s">
+      <c r="J23" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="53" t="s">
+      <c r="K23" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L23" s="53" t="s">
+      <c r="L23" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M23" s="22" t="s">
@@ -2128,18 +2059,18 @@
       <c r="U23" s="33"/>
     </row>
     <row r="24" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A24" s="60"/>
+      <c r="A24" s="49"/>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
       <c r="D24" s="25"/>
       <c r="E24" s="25"/>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="56"/>
-      <c r="J24" s="53"/>
-      <c r="K24" s="53"/>
-      <c r="L24" s="53"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="50"/>
+      <c r="J24" s="51"/>
+      <c r="K24" s="51"/>
+      <c r="L24" s="51"/>
       <c r="M24" s="22" t="s">
         <v>24</v>
       </c>
@@ -2149,18 +2080,18 @@
       <c r="R24" s="24"/>
     </row>
     <row r="25" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A25" s="60"/>
+      <c r="A25" s="49"/>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="D25" s="27"/>
       <c r="E25" s="27"/>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="56"/>
-      <c r="J25" s="53"/>
-      <c r="K25" s="53"/>
-      <c r="L25" s="53"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="51"/>
+      <c r="K25" s="51"/>
+      <c r="L25" s="51"/>
       <c r="M25" s="22" t="s">
         <v>25</v>
       </c>
@@ -2169,20 +2100,20 @@
       <c r="P25" s="34"/>
     </row>
     <row r="26" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A26" s="60"/>
+      <c r="A26" s="49"/>
       <c r="B26" s="21"/>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
       <c r="E26" s="21"/>
       <c r="F26" s="21"/>
       <c r="G26" s="21"/>
-      <c r="H26" s="56"/>
-      <c r="I26" s="56"/>
-      <c r="J26" s="54" t="s">
+      <c r="H26" s="50"/>
+      <c r="I26" s="50"/>
+      <c r="J26" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K26" s="54"/>
-      <c r="L26" s="54"/>
+      <c r="K26" s="52"/>
+      <c r="L26" s="52"/>
       <c r="M26" s="28" t="s">
         <v>27</v>
       </c>
@@ -2192,7 +2123,7 @@
       <c r="Q26" s="33"/>
     </row>
     <row r="27" spans="1:21" ht="9" customHeight="1">
-      <c r="A27" s="61"/>
+      <c r="A27" s="21"/>
       <c r="B27" s="29"/>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
@@ -2207,7 +2138,7 @@
       <c r="M27" s="31"/>
     </row>
     <row r="28" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A28" s="60">
+      <c r="A28" s="49">
         <v>5</v>
       </c>
       <c r="B28" s="25"/>
@@ -2216,19 +2147,19 @@
       <c r="E28" s="25"/>
       <c r="F28" s="21"/>
       <c r="G28" s="21"/>
-      <c r="H28" s="56" t="s">
+      <c r="H28" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="56" t="s">
+      <c r="I28" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="J28" s="53" t="s">
+      <c r="J28" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K28" s="53" t="s">
+      <c r="K28" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="L28" s="53" t="s">
+      <c r="L28" s="51" t="s">
         <v>22</v>
       </c>
       <c r="M28" s="22" t="s">
@@ -2239,18 +2170,18 @@
       <c r="P28" s="23"/>
     </row>
     <row r="29" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A29" s="60"/>
+      <c r="A29" s="49"/>
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
       <c r="E29" s="25"/>
       <c r="F29" s="20"/>
       <c r="G29" s="21"/>
-      <c r="H29" s="56"/>
-      <c r="I29" s="56"/>
-      <c r="J29" s="53"/>
-      <c r="K29" s="53"/>
-      <c r="L29" s="53"/>
+      <c r="H29" s="50"/>
+      <c r="I29" s="50"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="51"/>
+      <c r="L29" s="51"/>
       <c r="M29" s="22" t="s">
         <v>24</v>
       </c>
@@ -2259,18 +2190,18 @@
       <c r="P29" s="23"/>
     </row>
     <row r="30" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A30" s="60"/>
+      <c r="A30" s="49"/>
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
       <c r="D30" s="25"/>
       <c r="E30" s="25"/>
       <c r="F30" s="20"/>
       <c r="G30" s="21"/>
-      <c r="H30" s="56"/>
-      <c r="I30" s="56"/>
-      <c r="J30" s="53"/>
-      <c r="K30" s="53"/>
-      <c r="L30" s="53"/>
+      <c r="H30" s="50"/>
+      <c r="I30" s="50"/>
+      <c r="J30" s="51"/>
+      <c r="K30" s="51"/>
+      <c r="L30" s="51"/>
       <c r="M30" s="22" t="s">
         <v>25</v>
       </c>
@@ -2279,20 +2210,20 @@
       <c r="P30" s="23"/>
     </row>
     <row r="31" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A31" s="60"/>
+      <c r="A31" s="49"/>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
       <c r="D31" s="25"/>
       <c r="E31" s="25"/>
       <c r="F31" s="20"/>
       <c r="G31" s="21"/>
-      <c r="H31" s="56"/>
-      <c r="I31" s="56"/>
-      <c r="J31" s="54" t="s">
+      <c r="H31" s="50"/>
+      <c r="I31" s="50"/>
+      <c r="J31" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="K31" s="54"/>
-      <c r="L31" s="54"/>
+      <c r="K31" s="52"/>
+      <c r="L31" s="52"/>
       <c r="M31" s="28" t="s">
         <v>27</v>
       </c>
@@ -2301,7 +2232,7 @@
       <c r="P31" s="34"/>
     </row>
     <row r="32" spans="1:21" ht="18.75" hidden="1" customHeight="1">
-      <c r="A32" s="60"/>
+      <c r="A32" s="49"/>
       <c r="B32" s="35"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -2319,7 +2250,7 @@
       <c r="Q32" s="24"/>
     </row>
     <row r="33" spans="1:17" ht="18.75" hidden="1" customHeight="1">
-      <c r="A33" s="62"/>
+      <c r="A33" s="49"/>
       <c r="B33" s="35"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -2337,22 +2268,22 @@
     </row>
     <row r="34" spans="1:17" ht="36.75" customHeight="1">
       <c r="A34" s="21"/>
-      <c r="B34" s="57" t="s">
+      <c r="B34" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="57"/>
-      <c r="D34" s="57"/>
-      <c r="E34" s="57"/>
-      <c r="F34" s="57"/>
-      <c r="G34" s="57"/>
-      <c r="H34" s="57"/>
-      <c r="I34" s="58" t="s">
+      <c r="C34" s="47"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="47"/>
+      <c r="F34" s="47"/>
+      <c r="G34" s="47"/>
+      <c r="H34" s="47"/>
+      <c r="I34" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="58"/>
-      <c r="K34" s="58"/>
-      <c r="L34" s="58"/>
-      <c r="M34" s="58"/>
+      <c r="J34" s="48"/>
+      <c r="K34" s="48"/>
+      <c r="L34" s="48"/>
+      <c r="M34" s="48"/>
       <c r="Q34" s="33"/>
     </row>
     <row r="35" spans="1:17" ht="12.75" customHeight="1">
@@ -2378,15 +2309,27 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="I34:M34"/>
-    <mergeCell ref="A28:A33"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="I28:I31"/>
-    <mergeCell ref="J28:J30"/>
-    <mergeCell ref="K28:K30"/>
-    <mergeCell ref="L28:L30"/>
-    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="L13:L15"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="I8:I11"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="H13:H16"/>
+    <mergeCell ref="I13:I16"/>
+    <mergeCell ref="J13:J15"/>
+    <mergeCell ref="K13:K15"/>
     <mergeCell ref="L23:L25"/>
     <mergeCell ref="J26:L26"/>
     <mergeCell ref="A18:A21"/>
@@ -2401,31 +2344,19 @@
     <mergeCell ref="I23:I26"/>
     <mergeCell ref="J23:J25"/>
     <mergeCell ref="K23:K25"/>
-    <mergeCell ref="L13:L15"/>
-    <mergeCell ref="J16:L16"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="I8:I11"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="H13:H16"/>
-    <mergeCell ref="I13:I16"/>
-    <mergeCell ref="J13:J15"/>
-    <mergeCell ref="K13:K15"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="B34:H34"/>
+    <mergeCell ref="I34:M34"/>
+    <mergeCell ref="A28:A33"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="I28:I31"/>
+    <mergeCell ref="J28:J30"/>
+    <mergeCell ref="K28:K30"/>
+    <mergeCell ref="L28:L30"/>
+    <mergeCell ref="J31:L31"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19645669291338586" right="0.19645669291338586" top="0.11811023622047245" bottom="0.51181102362204722" header="0.11811023622047245" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="92" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -2436,11 +2367,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4F2601A-D0F9-4D66-91F1-48C323321E9D}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.796875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.19921875" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.19921875" style="2"/>
+    <col min="1" max="5" width="11.77734375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">
@@ -2525,11 +2456,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24971601-4DEF-44A8-8017-6E23A38D615F}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="12.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="11.796875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.19921875" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.19921875" style="2"/>
+    <col min="1" max="5" width="11.77734375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
Correction pb de build
</commit_message>
<xml_diff>
--- a/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
+++ b/src/main/resources/META-INF/resources/templates/Fiche-de-securite-template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seb/Documents/developpement-seb/santalina.nosync/src/main/resources/META-INF/resources/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seb/Documents/developpement-seb/santalina.nosync/src/main/webui/public/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C694601-994C-F748-BA42-0487CE74372D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756ADA97-08CD-4043-AC28-386E228E18F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="13900" xr2:uid="{0C40D413-3092-4696-A5DE-614A3C176F57}"/>
   </bookViews>
@@ -2425,7 +2425,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19645669291338586" right="0.19645669291338586" top="0.11811023622047245" bottom="0.51181102362204722" header="0.11811023622047245" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="92" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>